<commit_message>
Added pregnancy risk factors in visit summary
</commit_message>
<xml_diff>
--- a/forms/app/pregnancy.xlsx
+++ b/forms/app/pregnancy.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2437" uniqueCount="1426">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2477" uniqueCount="1432">
   <si>
     <t>type</t>
   </si>
@@ -4273,18 +4273,6 @@
     <t>previous_stillbirth_risk</t>
   </si>
   <si>
-    <t>delivery_complications_risk</t>
-  </si>
-  <si>
-    <t>selected(${delivery_complications},'prolonged_labor') or 
-selected(${delivery_complications},'large_perineal_tear') or 
-selected(${delivery_complications},'retained_placenta') or 
-selected(${delivery_complications},'aph') or 
-selected(${delivery_complications},'postpartum_hemorrage') or 
-selected(${delivery_complications},'enclampsia') or 
-selected(${delivery_complications},'big_baby')</t>
-  </si>
-  <si>
     <t xml:space="preserve">previous_miscarriage_risk </t>
   </si>
   <si>
@@ -4301,12 +4289,6 @@
   </si>
   <si>
     <t>big_baby_risk</t>
-  </si>
-  <si>
-    <t>Big Baby</t>
-  </si>
-  <si>
-    <t>selected(${big_baby},"yes")</t>
   </si>
   <si>
     <t>Malpresentation</t>
@@ -4328,12 +4310,6 @@
     <t>selected(${breech_position},"yes")</t>
   </si>
   <si>
-    <t>medical_conditions_risk</t>
-  </si>
-  <si>
-    <t xml:space="preserve">selected(${medical_conditions},"diabetes") or selected(${medical_conditions},"sickle_cell") or  selected(${medical_conditions},"cardiac_disease") </t>
-  </si>
-  <si>
     <t>Recommended to deliver at a higher level facility</t>
   </si>
   <si>
@@ -4420,9 +4396,6 @@
     <t xml:space="preserve">Kutarajia kuwa na mapacha </t>
   </si>
   <si>
-    <t xml:space="preserve">Kujifungua mtoto mkubwa ( zaidi ya kilo 4) (mimba hii au kabla) </t>
-  </si>
-  <si>
     <t>Milalo mibaya</t>
   </si>
   <si>
@@ -4445,21 +4418,6 @@
   </si>
   <si>
     <t>Hatari za kutumia dawa za mitishamba</t>
-  </si>
-  <si>
-    <t>${medical_conditions}</t>
-  </si>
-  <si>
-    <t>contains(${medical_conditions}, name) or name = 'none'</t>
-  </si>
-  <si>
-    <t>delivery_complications_risk_note</t>
-  </si>
-  <si>
-    <t xml:space="preserve">${delivery_complications_risk} </t>
-  </si>
-  <si>
-    <t>jr:choice-name(${delivery_complications}, '${delivery_complications}')</t>
   </si>
   <si>
     <t>${enabel} = "true"  and selected(${first_time_pregnant},'no') and ${previous_pregnancies} &gt; ${previous_miscarriages}</t>
@@ -4491,6 +4449,60 @@
   <si>
     <t xml:space="preserve">As soon as you are aware you are pregnant, it is important to go to the nearest health facility for antenatal care (ANC). You should go to ANC 8 times throughout your pregnancy as directed by the health worker.
 </t>
+  </si>
+  <si>
+    <t>prolonged_labor_risk</t>
+  </si>
+  <si>
+    <t>selected(${delivery_complications},'prolonged_labor')</t>
+  </si>
+  <si>
+    <t>selected(${delivery_complications},'large_perineal_tear')</t>
+  </si>
+  <si>
+    <t>selected(${delivery_complications},'retained_placenta')</t>
+  </si>
+  <si>
+    <t>selected(${delivery_complications},'aph')</t>
+  </si>
+  <si>
+    <t>selected(${delivery_complications},'postpartum_hemorrage')</t>
+  </si>
+  <si>
+    <t>selected(${delivery_complications},'enclampsia')</t>
+  </si>
+  <si>
+    <t>Uchungu wa muda mrefu ( Zaidi ya masaa 12)</t>
+  </si>
+  <si>
+    <t>large_perineal_tear_risk</t>
+  </si>
+  <si>
+    <t>retained_placenta_risk</t>
+  </si>
+  <si>
+    <t>aph_risk</t>
+  </si>
+  <si>
+    <t>postpartum_hemorrage_risk</t>
+  </si>
+  <si>
+    <t>enclampsia_risk</t>
+  </si>
+  <si>
+    <t>selected(${medical_conditions},"diabetes")</t>
+  </si>
+  <si>
+    <t>selected(${medical_conditions},"high_blood_pressure")</t>
+  </si>
+  <si>
+    <t>selected(${medical_conditions},"sickle_cell")</t>
+  </si>
+  <si>
+    <t>selected(${medical_conditions},"cardiac_disease")</t>
+  </si>
+  <si>
+    <t>selected(${delivery_complications},'big_baby') or selected(${big_baby},"yes")</t>
   </si>
 </sst>
 </file>
@@ -5109,7 +5121,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:Z332"/>
+  <dimension ref="A1:Z339"/>
   <sheetFormatPr defaultColWidth="14.40625" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="30.1328125" customWidth="1"/>
@@ -7612,10 +7624,10 @@
         <v>165</v>
       </c>
       <c r="C75" s="88" t="s">
-        <v>1425</v>
+        <v>1413</v>
       </c>
       <c r="D75" s="46" t="s">
-        <v>1424</v>
+        <v>1412</v>
       </c>
       <c r="E75" s="6"/>
       <c r="F75" s="4"/>
@@ -8658,7 +8670,7 @@
         <v>139</v>
       </c>
       <c r="F103" s="34" t="s">
-        <v>1416</v>
+        <v>1404</v>
       </c>
       <c r="G103" s="20"/>
       <c r="H103" s="8"/>
@@ -8698,7 +8710,7 @@
         <v>139</v>
       </c>
       <c r="F104" s="34" t="s">
-        <v>1417</v>
+        <v>1405</v>
       </c>
       <c r="G104" s="20"/>
       <c r="H104" s="8"/>
@@ -8738,7 +8750,7 @@
         <v>139</v>
       </c>
       <c r="F105" s="34" t="s">
-        <v>1418</v>
+        <v>1406</v>
       </c>
       <c r="G105" s="20"/>
       <c r="H105" s="8"/>
@@ -8824,7 +8836,7 @@
         <v>139</v>
       </c>
       <c r="F107" s="34" t="s">
-        <v>1416</v>
+        <v>1404</v>
       </c>
       <c r="G107" s="20"/>
       <c r="H107" s="8"/>
@@ -9098,7 +9110,7 @@
         <v>139</v>
       </c>
       <c r="F114" s="47" t="s">
-        <v>1419</v>
+        <v>1407</v>
       </c>
       <c r="G114" s="20"/>
       <c r="H114" s="8"/>
@@ -9920,7 +9932,7 @@
         <v>384</v>
       </c>
       <c r="D135" s="46" t="s">
-        <v>1422</v>
+        <v>1410</v>
       </c>
       <c r="E135" s="7" t="s">
         <v>139</v>
@@ -9960,9 +9972,11 @@
         <v>386</v>
       </c>
       <c r="D136" s="102" t="s">
-        <v>1421</v>
-      </c>
-      <c r="E136" s="20"/>
+        <v>1409</v>
+      </c>
+      <c r="E136" s="46" t="s">
+        <v>139</v>
+      </c>
       <c r="F136" s="34" t="s">
         <v>380</v>
       </c>
@@ -9998,9 +10012,11 @@
         <v>388</v>
       </c>
       <c r="D137" s="46" t="s">
-        <v>1423</v>
-      </c>
-      <c r="E137" s="20"/>
+        <v>1411</v>
+      </c>
+      <c r="E137" s="46" t="s">
+        <v>139</v>
+      </c>
       <c r="F137" s="34" t="s">
         <v>380</v>
       </c>
@@ -10038,7 +10054,9 @@
       <c r="D138" s="7" t="s">
         <v>293</v>
       </c>
-      <c r="E138" s="20"/>
+      <c r="E138" s="46" t="s">
+        <v>139</v>
+      </c>
       <c r="F138" s="34" t="s">
         <v>390</v>
       </c>
@@ -13806,7 +13824,7 @@
         <v>139</v>
       </c>
       <c r="F241" s="57" t="s">
-        <v>1420</v>
+        <v>1408</v>
       </c>
       <c r="G241" s="56"/>
       <c r="H241" s="56"/>
@@ -15695,7 +15713,7 @@
         <v>1346</v>
       </c>
       <c r="C303" s="88" t="s">
-        <v>1396</v>
+        <v>1390</v>
       </c>
       <c r="D303" s="46"/>
       <c r="F303" s="46"/>
@@ -15712,14 +15730,14 @@
         <v>1348</v>
       </c>
       <c r="D304" s="46" t="s">
-        <v>1397</v>
+        <v>1391</v>
       </c>
       <c r="F304" s="46" t="s">
         <v>1349</v>
       </c>
       <c r="G304" s="46"/>
     </row>
-    <row r="305" spans="1:26" s="87" customFormat="1" ht="13">
+    <row r="305" spans="1:12" s="87" customFormat="1" ht="13">
       <c r="A305" s="46" t="s">
         <v>109</v>
       </c>
@@ -15730,14 +15748,14 @@
         <v>1350</v>
       </c>
       <c r="D305" s="101" t="s">
-        <v>1398</v>
+        <v>1392</v>
       </c>
       <c r="F305" s="46" t="s">
         <v>1352</v>
       </c>
       <c r="G305" s="46"/>
     </row>
-    <row r="306" spans="1:26" s="87" customFormat="1" ht="13">
+    <row r="306" spans="1:12" s="87" customFormat="1" ht="13">
       <c r="A306" s="46" t="s">
         <v>109</v>
       </c>
@@ -15748,507 +15766,403 @@
         <v>1353</v>
       </c>
       <c r="D306" s="101" t="s">
-        <v>1399</v>
+        <v>1393</v>
       </c>
       <c r="F306" s="46" t="s">
         <v>1354</v>
       </c>
       <c r="G306" s="46"/>
     </row>
-    <row r="307" spans="1:26" s="87" customFormat="1" ht="19.75" customHeight="1">
+    <row r="307" spans="1:12" s="87" customFormat="1" ht="19.75" customHeight="1">
       <c r="A307" s="46" t="s">
-        <v>41</v>
+        <v>109</v>
       </c>
       <c r="B307" s="46" t="s">
-        <v>1356</v>
-      </c>
-      <c r="C307" s="88"/>
-      <c r="D307" s="88"/>
+        <v>1414</v>
+      </c>
+      <c r="C307" s="46" t="s">
+        <v>1276</v>
+      </c>
+      <c r="D307" s="46" t="s">
+        <v>1421</v>
+      </c>
       <c r="F307" s="88" t="s">
-        <v>1357</v>
+        <v>1415</v>
       </c>
       <c r="G307" s="46"/>
-      <c r="L307" s="101" t="s">
-        <v>1415</v>
-      </c>
-    </row>
-    <row r="308" spans="1:26" s="97" customFormat="1" ht="19.75" customHeight="1">
+      <c r="L307" s="101"/>
+    </row>
+    <row r="308" spans="1:12" s="97" customFormat="1" ht="19.75" customHeight="1">
       <c r="A308" s="46" t="s">
         <v>109</v>
       </c>
       <c r="B308" s="46" t="s">
-        <v>1413</v>
-      </c>
-      <c r="C308" s="88" t="s">
-        <v>1414</v>
-      </c>
-      <c r="D308" s="88"/>
-      <c r="F308" s="88"/>
+        <v>1422</v>
+      </c>
+      <c r="C308" s="46" t="s">
+        <v>1279</v>
+      </c>
+      <c r="D308" s="46" t="s">
+        <v>1280</v>
+      </c>
+      <c r="F308" s="88" t="s">
+        <v>1416</v>
+      </c>
       <c r="G308" s="46"/>
       <c r="L308" s="101"/>
     </row>
-    <row r="309" spans="1:26" s="87" customFormat="1" ht="13">
+    <row r="309" spans="1:12" s="97" customFormat="1" ht="19.75" customHeight="1">
       <c r="A309" s="46" t="s">
         <v>109</v>
       </c>
       <c r="B309" s="46" t="s">
-        <v>1358</v>
-      </c>
-      <c r="C309" s="88" t="s">
-        <v>1359</v>
-      </c>
-      <c r="D309" s="101" t="s">
-        <v>1400</v>
-      </c>
-      <c r="F309" s="46" t="s">
-        <v>255</v>
+        <v>1423</v>
+      </c>
+      <c r="C309" s="46" t="s">
+        <v>1282</v>
+      </c>
+      <c r="D309" s="46" t="s">
+        <v>1283</v>
+      </c>
+      <c r="F309" s="88" t="s">
+        <v>1417</v>
       </c>
       <c r="G309" s="46"/>
-    </row>
-    <row r="310" spans="1:26" s="87" customFormat="1" ht="13">
+      <c r="L309" s="101"/>
+    </row>
+    <row r="310" spans="1:12" s="97" customFormat="1" ht="19.75" customHeight="1">
       <c r="A310" s="46" t="s">
         <v>109</v>
       </c>
       <c r="B310" s="46" t="s">
-        <v>1360</v>
-      </c>
-      <c r="C310" s="88" t="s">
-        <v>1361</v>
-      </c>
-      <c r="D310" s="101" t="s">
-        <v>1401</v>
-      </c>
-      <c r="F310" s="46" t="s">
-        <v>1362</v>
+        <v>1424</v>
+      </c>
+      <c r="C310" s="46" t="s">
+        <v>1285</v>
+      </c>
+      <c r="D310" s="46" t="s">
+        <v>1286</v>
+      </c>
+      <c r="F310" s="88" t="s">
+        <v>1418</v>
       </c>
       <c r="G310" s="46"/>
-    </row>
-    <row r="311" spans="1:26" s="87" customFormat="1" ht="13">
+      <c r="L310" s="101"/>
+    </row>
+    <row r="311" spans="1:12" s="97" customFormat="1" ht="19.75" customHeight="1">
       <c r="A311" s="46" t="s">
         <v>109</v>
       </c>
       <c r="B311" s="46" t="s">
-        <v>1363</v>
-      </c>
-      <c r="C311" s="88" t="s">
-        <v>1364</v>
-      </c>
-      <c r="D311" s="101" t="s">
-        <v>1402</v>
-      </c>
-      <c r="F311" s="46" t="s">
-        <v>1365</v>
+        <v>1425</v>
+      </c>
+      <c r="C311" s="46" t="s">
+        <v>1288</v>
+      </c>
+      <c r="D311" s="46" t="s">
+        <v>1289</v>
+      </c>
+      <c r="F311" s="88" t="s">
+        <v>1419</v>
       </c>
       <c r="G311" s="46"/>
-    </row>
-    <row r="312" spans="1:26" s="87" customFormat="1" ht="13">
+      <c r="L311" s="101"/>
+    </row>
+    <row r="312" spans="1:12" s="97" customFormat="1" ht="19.75" customHeight="1">
       <c r="A312" s="46" t="s">
         <v>109</v>
       </c>
       <c r="B312" s="46" t="s">
-        <v>1369</v>
-      </c>
-      <c r="C312" s="88" t="s">
-        <v>1366</v>
-      </c>
-      <c r="D312" s="101" t="s">
-        <v>1403</v>
-      </c>
-      <c r="F312" s="46" t="s">
-        <v>1367</v>
+        <v>1426</v>
+      </c>
+      <c r="C312" s="46" t="s">
+        <v>1291</v>
+      </c>
+      <c r="D312" s="46" t="s">
+        <v>446</v>
+      </c>
+      <c r="F312" s="88" t="s">
+        <v>1420</v>
       </c>
       <c r="G312" s="46"/>
-    </row>
-    <row r="313" spans="1:26" s="87" customFormat="1" ht="26">
+      <c r="L312" s="101"/>
+    </row>
+    <row r="313" spans="1:12" s="97" customFormat="1" ht="19.75" customHeight="1">
       <c r="A313" s="46" t="s">
         <v>109</v>
       </c>
-      <c r="B313" s="88" t="s">
-        <v>1370</v>
-      </c>
-      <c r="C313" s="88" t="s">
-        <v>1368</v>
-      </c>
-      <c r="D313" s="101" t="s">
-        <v>1404</v>
-      </c>
-      <c r="F313" s="46" t="s">
-        <v>1371</v>
+      <c r="B313" s="46" t="s">
+        <v>1361</v>
+      </c>
+      <c r="C313" s="46" t="s">
+        <v>1292</v>
+      </c>
+      <c r="D313" s="46" t="s">
+        <v>1293</v>
+      </c>
+      <c r="F313" s="88" t="s">
+        <v>1431</v>
       </c>
       <c r="G313" s="46"/>
-    </row>
-    <row r="314" spans="1:26" s="87" customFormat="1" ht="13">
+      <c r="L313" s="101"/>
+    </row>
+    <row r="314" spans="1:12" s="87" customFormat="1" ht="13">
       <c r="A314" s="46" t="s">
         <v>109</v>
       </c>
       <c r="B314" s="46" t="s">
-        <v>1372</v>
+        <v>1356</v>
       </c>
       <c r="C314" s="88" t="s">
-        <v>1411</v>
-      </c>
-      <c r="D314" s="88" t="s">
-        <v>1411</v>
+        <v>1357</v>
+      </c>
+      <c r="D314" s="101" t="s">
+        <v>1394</v>
       </c>
       <c r="F314" s="46" t="s">
-        <v>1373</v>
+        <v>255</v>
       </c>
       <c r="G314" s="46"/>
-      <c r="M314" s="101" t="s">
-        <v>1412</v>
-      </c>
-    </row>
-    <row r="315" spans="1:26" s="87" customFormat="1" ht="13">
+    </row>
+    <row r="315" spans="1:12" s="87" customFormat="1" ht="13">
       <c r="A315" s="46" t="s">
         <v>109</v>
       </c>
       <c r="B315" s="46" t="s">
-        <v>1383</v>
+        <v>1358</v>
       </c>
       <c r="C315" s="88" t="s">
-        <v>1374</v>
+        <v>1359</v>
       </c>
       <c r="D315" s="101" t="s">
-        <v>1405</v>
+        <v>1395</v>
       </c>
       <c r="F315" s="46" t="s">
-        <v>1375</v>
+        <v>1360</v>
       </c>
       <c r="G315" s="46"/>
     </row>
-    <row r="316" spans="1:26" s="87" customFormat="1" ht="13">
+    <row r="316" spans="1:12" s="87" customFormat="1" ht="13">
       <c r="A316" s="46" t="s">
         <v>109</v>
       </c>
       <c r="B316" s="46" t="s">
-        <v>1394</v>
+        <v>1365</v>
       </c>
       <c r="C316" s="88" t="s">
-        <v>1406</v>
+        <v>1362</v>
       </c>
       <c r="D316" s="101" t="s">
-        <v>1407</v>
+        <v>1396</v>
       </c>
       <c r="F316" s="46" t="s">
-        <v>1376</v>
+        <v>1363</v>
       </c>
       <c r="G316" s="46"/>
     </row>
-    <row r="317" spans="1:26" s="87" customFormat="1" ht="13">
+    <row r="317" spans="1:12" s="87" customFormat="1" ht="26">
       <c r="A317" s="46" t="s">
         <v>109</v>
       </c>
-      <c r="B317" s="46" t="s">
-        <v>1391</v>
+      <c r="B317" s="88" t="s">
+        <v>1366</v>
       </c>
       <c r="C317" s="88" t="s">
-        <v>1377</v>
+        <v>1364</v>
       </c>
       <c r="D317" s="101" t="s">
-        <v>1408</v>
+        <v>1397</v>
       </c>
       <c r="F317" s="46" t="s">
-        <v>1378</v>
+        <v>1367</v>
       </c>
       <c r="G317" s="46"/>
     </row>
-    <row r="318" spans="1:26" s="91" customFormat="1" ht="13">
+    <row r="318" spans="1:12" s="97" customFormat="1" ht="13">
       <c r="A318" s="46" t="s">
         <v>109</v>
       </c>
       <c r="B318" s="46" t="s">
-        <v>1392</v>
-      </c>
-      <c r="C318" s="88" t="s">
-        <v>1380</v>
-      </c>
-      <c r="D318" s="101" t="s">
-        <v>1409</v>
+        <v>1295</v>
+      </c>
+      <c r="C318" s="46" t="s">
+        <v>1296</v>
+      </c>
+      <c r="D318" s="46" t="s">
+        <v>1297</v>
       </c>
       <c r="F318" s="46" t="s">
-        <v>1382</v>
+        <v>1428</v>
       </c>
       <c r="G318" s="46"/>
     </row>
-    <row r="319" spans="1:26" s="91" customFormat="1" ht="13">
+    <row r="319" spans="1:12" s="97" customFormat="1" ht="13">
       <c r="A319" s="46" t="s">
         <v>109</v>
       </c>
       <c r="B319" s="46" t="s">
-        <v>1393</v>
-      </c>
-      <c r="C319" s="88" t="s">
+        <v>1298</v>
+      </c>
+      <c r="C319" s="46" t="s">
+        <v>1299</v>
+      </c>
+      <c r="D319" s="46" t="s">
+        <v>1300</v>
+      </c>
+      <c r="F319" s="46" t="s">
+        <v>1427</v>
+      </c>
+      <c r="G319" s="46"/>
+    </row>
+    <row r="320" spans="1:12" s="97" customFormat="1" ht="13">
+      <c r="A320" s="46" t="s">
+        <v>109</v>
+      </c>
+      <c r="B320" s="46" t="s">
+        <v>1301</v>
+      </c>
+      <c r="C320" s="46" t="s">
+        <v>1302</v>
+      </c>
+      <c r="D320" s="46" t="s">
+        <v>1303</v>
+      </c>
+      <c r="F320" s="46" t="s">
+        <v>1429</v>
+      </c>
+      <c r="G320" s="46"/>
+    </row>
+    <row r="321" spans="1:26" s="97" customFormat="1" ht="13">
+      <c r="A321" s="46" t="s">
+        <v>109</v>
+      </c>
+      <c r="B321" s="46" t="s">
+        <v>1304</v>
+      </c>
+      <c r="C321" s="46" t="s">
+        <v>1305</v>
+      </c>
+      <c r="D321" s="46" t="s">
+        <v>1306</v>
+      </c>
+      <c r="F321" s="46" t="s">
+        <v>1430</v>
+      </c>
+      <c r="G321" s="46"/>
+    </row>
+    <row r="322" spans="1:26" s="87" customFormat="1" ht="13">
+      <c r="A322" s="46" t="s">
+        <v>109</v>
+      </c>
+      <c r="B322" s="46" t="s">
+        <v>1377</v>
+      </c>
+      <c r="C322" s="88" t="s">
+        <v>1368</v>
+      </c>
+      <c r="D322" s="101" t="s">
+        <v>1398</v>
+      </c>
+      <c r="F322" s="46" t="s">
+        <v>1369</v>
+      </c>
+      <c r="G322" s="46"/>
+    </row>
+    <row r="323" spans="1:26" s="87" customFormat="1" ht="13">
+      <c r="A323" s="46" t="s">
+        <v>109</v>
+      </c>
+      <c r="B323" s="46" t="s">
+        <v>1388</v>
+      </c>
+      <c r="C323" s="88" t="s">
+        <v>1399</v>
+      </c>
+      <c r="D323" s="101" t="s">
+        <v>1400</v>
+      </c>
+      <c r="F323" s="46" t="s">
+        <v>1370</v>
+      </c>
+      <c r="G323" s="46"/>
+    </row>
+    <row r="324" spans="1:26" s="87" customFormat="1" ht="13">
+      <c r="A324" s="46" t="s">
+        <v>109</v>
+      </c>
+      <c r="B324" s="46" t="s">
+        <v>1385</v>
+      </c>
+      <c r="C324" s="88" t="s">
+        <v>1371</v>
+      </c>
+      <c r="D324" s="101" t="s">
+        <v>1401</v>
+      </c>
+      <c r="F324" s="46" t="s">
+        <v>1372</v>
+      </c>
+      <c r="G324" s="46"/>
+    </row>
+    <row r="325" spans="1:26" s="91" customFormat="1" ht="13">
+      <c r="A325" s="46" t="s">
+        <v>109</v>
+      </c>
+      <c r="B325" s="46" t="s">
+        <v>1386</v>
+      </c>
+      <c r="C325" s="88" t="s">
+        <v>1374</v>
+      </c>
+      <c r="D325" s="101" t="s">
+        <v>1402</v>
+      </c>
+      <c r="F325" s="46" t="s">
+        <v>1376</v>
+      </c>
+      <c r="G325" s="46"/>
+    </row>
+    <row r="326" spans="1:26" s="91" customFormat="1" ht="13">
+      <c r="A326" s="46" t="s">
+        <v>109</v>
+      </c>
+      <c r="B326" s="46" t="s">
+        <v>1387</v>
+      </c>
+      <c r="C326" s="88" t="s">
+        <v>1373</v>
+      </c>
+      <c r="D326" s="101" t="s">
+        <v>1403</v>
+      </c>
+      <c r="F326" s="46" t="s">
+        <v>1375</v>
+      </c>
+      <c r="G326" s="46"/>
+    </row>
+    <row r="327" spans="1:26" s="87" customFormat="1" ht="26">
+      <c r="A327" s="92" t="s">
+        <v>109</v>
+      </c>
+      <c r="B327" s="92" t="s">
+        <v>831</v>
+      </c>
+      <c r="C327" s="92" t="s">
+        <v>1378</v>
+      </c>
+      <c r="D327" s="93" t="s">
         <v>1379</v>
       </c>
-      <c r="D319" s="101" t="s">
-        <v>1410</v>
-      </c>
-      <c r="F319" s="46" t="s">
-        <v>1381</v>
-      </c>
-      <c r="G319" s="46"/>
-    </row>
-    <row r="320" spans="1:26" s="87" customFormat="1" ht="26">
-      <c r="A320" s="92" t="s">
-        <v>109</v>
-      </c>
-      <c r="B320" s="92" t="s">
-        <v>831</v>
-      </c>
-      <c r="C320" s="92" t="s">
-        <v>1384</v>
-      </c>
-      <c r="D320" s="93" t="s">
-        <v>1385</v>
-      </c>
-      <c r="E320" s="92"/>
-      <c r="F320" s="93" t="s">
-        <v>1386</v>
-      </c>
-      <c r="G320" s="92"/>
-      <c r="H320" s="92"/>
-      <c r="I320" s="92"/>
-      <c r="J320" s="92"/>
-      <c r="K320" s="92"/>
-      <c r="L320" s="92"/>
-      <c r="M320" s="92"/>
-      <c r="N320" s="92"/>
-      <c r="O320" s="92"/>
-      <c r="P320" s="92"/>
-      <c r="Q320" s="92"/>
-      <c r="R320" s="92"/>
-      <c r="S320" s="92"/>
-      <c r="T320" s="92"/>
-      <c r="U320" s="92"/>
-      <c r="V320" s="92"/>
-      <c r="W320" s="92"/>
-      <c r="X320" s="92"/>
-      <c r="Y320" s="92"/>
-      <c r="Z320" s="92"/>
-    </row>
-    <row r="321" spans="1:26" s="87" customFormat="1" ht="13">
-      <c r="A321" s="92" t="s">
-        <v>109</v>
-      </c>
-      <c r="B321" s="92" t="s">
-        <v>832</v>
-      </c>
-      <c r="C321" s="92" t="s">
-        <v>1395</v>
-      </c>
-      <c r="D321" s="93" t="s">
-        <v>833</v>
-      </c>
-      <c r="E321" s="92"/>
-      <c r="F321" s="92" t="s">
-        <v>834</v>
-      </c>
-      <c r="G321" s="92"/>
-      <c r="H321" s="92"/>
-      <c r="I321" s="92"/>
-      <c r="J321" s="92"/>
-      <c r="K321" s="92"/>
-      <c r="L321" s="92"/>
-      <c r="M321" s="92"/>
-      <c r="N321" s="92"/>
-      <c r="O321" s="92"/>
-      <c r="P321" s="92"/>
-      <c r="Q321" s="92"/>
-      <c r="R321" s="92"/>
-      <c r="S321" s="92"/>
-      <c r="T321" s="92"/>
-      <c r="U321" s="92"/>
-      <c r="V321" s="92"/>
-      <c r="W321" s="92"/>
-      <c r="X321" s="92"/>
-      <c r="Y321" s="92"/>
-      <c r="Z321" s="92"/>
-    </row>
-    <row r="322" spans="1:26" ht="13">
-      <c r="A322" s="92" t="s">
-        <v>109</v>
-      </c>
-      <c r="B322" s="92" t="s">
-        <v>835</v>
-      </c>
-      <c r="C322" s="92" t="s">
-        <v>836</v>
-      </c>
-      <c r="D322" s="94" t="s">
-        <v>837</v>
-      </c>
-      <c r="E322" s="92"/>
-      <c r="F322" s="95" t="s">
-        <v>838</v>
-      </c>
-      <c r="G322" s="92" t="s">
-        <v>839</v>
-      </c>
-      <c r="H322" s="92"/>
-      <c r="I322" s="92"/>
-      <c r="J322" s="92"/>
-      <c r="K322" s="92"/>
-      <c r="L322" s="92"/>
-      <c r="M322" s="92"/>
-      <c r="N322" s="92"/>
-      <c r="O322" s="92"/>
-      <c r="P322" s="92"/>
-      <c r="Q322" s="92"/>
-      <c r="R322" s="92"/>
-      <c r="S322" s="92"/>
-      <c r="T322" s="92"/>
-      <c r="U322" s="92"/>
-      <c r="V322" s="92"/>
-      <c r="W322" s="92"/>
-      <c r="X322" s="92"/>
-      <c r="Y322" s="92"/>
-      <c r="Z322" s="92"/>
-    </row>
-    <row r="323" spans="1:26" ht="28.5">
-      <c r="A323" s="92" t="s">
-        <v>109</v>
-      </c>
-      <c r="B323" s="92" t="s">
-        <v>840</v>
-      </c>
-      <c r="C323" s="92" t="s">
-        <v>1387</v>
-      </c>
-      <c r="D323" s="92" t="s">
-        <v>1388</v>
-      </c>
-      <c r="E323" s="92"/>
-      <c r="F323" s="96" t="s">
-        <v>1389</v>
-      </c>
-      <c r="G323" s="92" t="s">
-        <v>839</v>
-      </c>
-      <c r="H323" s="92"/>
-      <c r="I323" s="92"/>
-      <c r="J323" s="92"/>
-      <c r="K323" s="92"/>
-      <c r="L323" s="92"/>
-      <c r="M323" s="92"/>
-      <c r="N323" s="92"/>
-      <c r="O323" s="92"/>
-      <c r="P323" s="92"/>
-      <c r="Q323" s="92"/>
-      <c r="R323" s="92"/>
-      <c r="S323" s="92"/>
-      <c r="T323" s="92"/>
-      <c r="U323" s="92"/>
-      <c r="V323" s="92"/>
-      <c r="W323" s="92"/>
-      <c r="X323" s="92"/>
-      <c r="Y323" s="92"/>
-      <c r="Z323" s="92"/>
-    </row>
-    <row r="324" spans="1:26" ht="13">
-      <c r="A324" s="92" t="s">
-        <v>109</v>
-      </c>
-      <c r="B324" s="92" t="s">
-        <v>841</v>
-      </c>
-      <c r="C324" s="92" t="s">
-        <v>1390</v>
-      </c>
-      <c r="D324" s="93" t="s">
-        <v>842</v>
-      </c>
-      <c r="E324" s="92"/>
-      <c r="F324" s="92" t="s">
-        <v>843</v>
-      </c>
-      <c r="G324" s="92" t="s">
-        <v>839</v>
-      </c>
-      <c r="H324" s="92"/>
-      <c r="I324" s="92"/>
-      <c r="J324" s="92"/>
-      <c r="K324" s="92"/>
-      <c r="L324" s="92"/>
-      <c r="M324" s="92"/>
-      <c r="N324" s="92"/>
-      <c r="O324" s="92"/>
-      <c r="P324" s="92"/>
-      <c r="Q324" s="92"/>
-      <c r="R324" s="92"/>
-      <c r="S324" s="92"/>
-      <c r="T324" s="92"/>
-      <c r="U324" s="92"/>
-      <c r="V324" s="92"/>
-      <c r="W324" s="92"/>
-      <c r="X324" s="92"/>
-      <c r="Y324" s="92"/>
-      <c r="Z324" s="92"/>
-    </row>
-    <row r="325" spans="1:26" s="89" customFormat="1" ht="13">
-      <c r="A325" s="46" t="s">
-        <v>113</v>
-      </c>
-      <c r="B325" s="46" t="s">
-        <v>827</v>
-      </c>
-      <c r="C325" s="46"/>
-      <c r="D325" s="46"/>
-      <c r="F325" s="46"/>
-      <c r="G325" s="46"/>
-    </row>
-    <row r="326" spans="1:26" s="89" customFormat="1" ht="25.5" customHeight="1">
-      <c r="A326" s="92" t="s">
-        <v>41</v>
-      </c>
-      <c r="B326" s="92" t="s">
-        <v>844</v>
-      </c>
-      <c r="C326" s="92"/>
-      <c r="D326" s="92"/>
-      <c r="E326" s="92"/>
-      <c r="F326" s="92"/>
-      <c r="G326" s="92"/>
-      <c r="H326" s="92"/>
-      <c r="I326" s="92"/>
-      <c r="J326" s="92"/>
-      <c r="K326" s="92"/>
-      <c r="L326" s="92" t="s">
-        <v>845</v>
-      </c>
-      <c r="M326" s="92"/>
-      <c r="N326" s="92"/>
-      <c r="O326" s="92"/>
-      <c r="P326" s="92"/>
-      <c r="Q326" s="92"/>
-      <c r="R326" s="92"/>
-      <c r="S326" s="92"/>
-      <c r="T326" s="92"/>
-      <c r="U326" s="92"/>
-      <c r="V326" s="92"/>
-      <c r="W326" s="92"/>
-      <c r="X326" s="92"/>
-      <c r="Y326" s="92"/>
-      <c r="Z326" s="92"/>
-    </row>
-    <row r="327" spans="1:26" ht="13">
-      <c r="A327" s="92" t="s">
-        <v>41</v>
-      </c>
-      <c r="B327" s="92" t="s">
-        <v>846</v>
-      </c>
-      <c r="C327" s="92"/>
-      <c r="D327" s="92"/>
       <c r="E327" s="92"/>
-      <c r="F327" s="92"/>
+      <c r="F327" s="93" t="s">
+        <v>1380</v>
+      </c>
       <c r="G327" s="92"/>
       <c r="H327" s="92"/>
       <c r="I327" s="92"/>
       <c r="J327" s="92"/>
       <c r="K327" s="92"/>
-      <c r="L327" s="92" t="s">
-        <v>847</v>
-      </c>
+      <c r="L327" s="92"/>
       <c r="M327" s="92"/>
       <c r="N327" s="92"/>
       <c r="O327" s="92"/>
@@ -16264,25 +16178,29 @@
       <c r="Y327" s="92"/>
       <c r="Z327" s="92"/>
     </row>
-    <row r="328" spans="1:26" ht="13">
+    <row r="328" spans="1:26" s="87" customFormat="1" ht="13">
       <c r="A328" s="92" t="s">
-        <v>41</v>
+        <v>109</v>
       </c>
       <c r="B328" s="92" t="s">
-        <v>848</v>
-      </c>
-      <c r="C328" s="92"/>
-      <c r="D328" s="92"/>
+        <v>832</v>
+      </c>
+      <c r="C328" s="92" t="s">
+        <v>1389</v>
+      </c>
+      <c r="D328" s="93" t="s">
+        <v>833</v>
+      </c>
       <c r="E328" s="92"/>
-      <c r="F328" s="92"/>
+      <c r="F328" s="92" t="s">
+        <v>834</v>
+      </c>
       <c r="G328" s="92"/>
       <c r="H328" s="92"/>
       <c r="I328" s="92"/>
       <c r="J328" s="92"/>
       <c r="K328" s="92"/>
-      <c r="L328" s="92" t="s">
-        <v>849</v>
-      </c>
+      <c r="L328" s="92"/>
       <c r="M328" s="92"/>
       <c r="N328" s="92"/>
       <c r="O328" s="92"/>
@@ -16300,23 +16218,29 @@
     </row>
     <row r="329" spans="1:26" ht="13">
       <c r="A329" s="92" t="s">
-        <v>41</v>
+        <v>109</v>
       </c>
       <c r="B329" s="92" t="s">
-        <v>850</v>
-      </c>
-      <c r="C329" s="92"/>
-      <c r="D329" s="92"/>
+        <v>835</v>
+      </c>
+      <c r="C329" s="92" t="s">
+        <v>836</v>
+      </c>
+      <c r="D329" s="94" t="s">
+        <v>837</v>
+      </c>
       <c r="E329" s="92"/>
-      <c r="F329" s="92"/>
-      <c r="G329" s="92"/>
+      <c r="F329" s="95" t="s">
+        <v>838</v>
+      </c>
+      <c r="G329" s="92" t="s">
+        <v>839</v>
+      </c>
       <c r="H329" s="92"/>
       <c r="I329" s="92"/>
       <c r="J329" s="92"/>
       <c r="K329" s="92"/>
-      <c r="L329" s="92" t="s">
-        <v>851</v>
-      </c>
+      <c r="L329" s="92"/>
       <c r="M329" s="92"/>
       <c r="N329" s="92"/>
       <c r="O329" s="92"/>
@@ -16332,25 +16256,31 @@
       <c r="Y329" s="92"/>
       <c r="Z329" s="92"/>
     </row>
-    <row r="330" spans="1:26" ht="13">
+    <row r="330" spans="1:26" ht="28.5">
       <c r="A330" s="92" t="s">
-        <v>41</v>
+        <v>109</v>
       </c>
       <c r="B330" s="92" t="s">
-        <v>852</v>
-      </c>
-      <c r="C330" s="92"/>
-      <c r="D330" s="92"/>
+        <v>840</v>
+      </c>
+      <c r="C330" s="92" t="s">
+        <v>1381</v>
+      </c>
+      <c r="D330" s="92" t="s">
+        <v>1382</v>
+      </c>
       <c r="E330" s="92"/>
-      <c r="F330" s="92"/>
-      <c r="G330" s="92"/>
+      <c r="F330" s="96" t="s">
+        <v>1383</v>
+      </c>
+      <c r="G330" s="92" t="s">
+        <v>839</v>
+      </c>
       <c r="H330" s="92"/>
       <c r="I330" s="92"/>
       <c r="J330" s="92"/>
       <c r="K330" s="92"/>
-      <c r="L330" s="92" t="s">
-        <v>853</v>
-      </c>
+      <c r="L330" s="92"/>
       <c r="M330" s="92"/>
       <c r="N330" s="92"/>
       <c r="O330" s="92"/>
@@ -16367,12 +16297,234 @@
       <c r="Z330" s="92"/>
     </row>
     <row r="331" spans="1:26" ht="13">
-      <c r="A331" s="2"/>
-      <c r="L331" s="2"/>
-    </row>
-    <row r="332" spans="1:26" ht="13">
-      <c r="A332" s="2"/>
-      <c r="L332" s="2"/>
+      <c r="A331" s="92" t="s">
+        <v>109</v>
+      </c>
+      <c r="B331" s="92" t="s">
+        <v>841</v>
+      </c>
+      <c r="C331" s="92" t="s">
+        <v>1384</v>
+      </c>
+      <c r="D331" s="93" t="s">
+        <v>842</v>
+      </c>
+      <c r="E331" s="92"/>
+      <c r="F331" s="92" t="s">
+        <v>843</v>
+      </c>
+      <c r="G331" s="92" t="s">
+        <v>839</v>
+      </c>
+      <c r="H331" s="92"/>
+      <c r="I331" s="92"/>
+      <c r="J331" s="92"/>
+      <c r="K331" s="92"/>
+      <c r="L331" s="92"/>
+      <c r="M331" s="92"/>
+      <c r="N331" s="92"/>
+      <c r="O331" s="92"/>
+      <c r="P331" s="92"/>
+      <c r="Q331" s="92"/>
+      <c r="R331" s="92"/>
+      <c r="S331" s="92"/>
+      <c r="T331" s="92"/>
+      <c r="U331" s="92"/>
+      <c r="V331" s="92"/>
+      <c r="W331" s="92"/>
+      <c r="X331" s="92"/>
+      <c r="Y331" s="92"/>
+      <c r="Z331" s="92"/>
+    </row>
+    <row r="332" spans="1:26" s="89" customFormat="1" ht="13">
+      <c r="A332" s="46" t="s">
+        <v>113</v>
+      </c>
+      <c r="B332" s="46" t="s">
+        <v>827</v>
+      </c>
+      <c r="C332" s="46"/>
+      <c r="D332" s="46"/>
+      <c r="F332" s="46"/>
+      <c r="G332" s="46"/>
+    </row>
+    <row r="333" spans="1:26" s="89" customFormat="1" ht="25.5" customHeight="1">
+      <c r="A333" s="92" t="s">
+        <v>41</v>
+      </c>
+      <c r="B333" s="92" t="s">
+        <v>844</v>
+      </c>
+      <c r="C333" s="92"/>
+      <c r="D333" s="92"/>
+      <c r="E333" s="92"/>
+      <c r="F333" s="92"/>
+      <c r="G333" s="92"/>
+      <c r="H333" s="92"/>
+      <c r="I333" s="92"/>
+      <c r="J333" s="92"/>
+      <c r="K333" s="92"/>
+      <c r="L333" s="92" t="s">
+        <v>845</v>
+      </c>
+      <c r="M333" s="92"/>
+      <c r="N333" s="92"/>
+      <c r="O333" s="92"/>
+      <c r="P333" s="92"/>
+      <c r="Q333" s="92"/>
+      <c r="R333" s="92"/>
+      <c r="S333" s="92"/>
+      <c r="T333" s="92"/>
+      <c r="U333" s="92"/>
+      <c r="V333" s="92"/>
+      <c r="W333" s="92"/>
+      <c r="X333" s="92"/>
+      <c r="Y333" s="92"/>
+      <c r="Z333" s="92"/>
+    </row>
+    <row r="334" spans="1:26" ht="13">
+      <c r="A334" s="92" t="s">
+        <v>41</v>
+      </c>
+      <c r="B334" s="92" t="s">
+        <v>846</v>
+      </c>
+      <c r="C334" s="92"/>
+      <c r="D334" s="92"/>
+      <c r="E334" s="92"/>
+      <c r="F334" s="92"/>
+      <c r="G334" s="92"/>
+      <c r="H334" s="92"/>
+      <c r="I334" s="92"/>
+      <c r="J334" s="92"/>
+      <c r="K334" s="92"/>
+      <c r="L334" s="92" t="s">
+        <v>847</v>
+      </c>
+      <c r="M334" s="92"/>
+      <c r="N334" s="92"/>
+      <c r="O334" s="92"/>
+      <c r="P334" s="92"/>
+      <c r="Q334" s="92"/>
+      <c r="R334" s="92"/>
+      <c r="S334" s="92"/>
+      <c r="T334" s="92"/>
+      <c r="U334" s="92"/>
+      <c r="V334" s="92"/>
+      <c r="W334" s="92"/>
+      <c r="X334" s="92"/>
+      <c r="Y334" s="92"/>
+      <c r="Z334" s="92"/>
+    </row>
+    <row r="335" spans="1:26" ht="13">
+      <c r="A335" s="92" t="s">
+        <v>41</v>
+      </c>
+      <c r="B335" s="92" t="s">
+        <v>848</v>
+      </c>
+      <c r="C335" s="92"/>
+      <c r="D335" s="92"/>
+      <c r="E335" s="92"/>
+      <c r="F335" s="92"/>
+      <c r="G335" s="92"/>
+      <c r="H335" s="92"/>
+      <c r="I335" s="92"/>
+      <c r="J335" s="92"/>
+      <c r="K335" s="92"/>
+      <c r="L335" s="92" t="s">
+        <v>849</v>
+      </c>
+      <c r="M335" s="92"/>
+      <c r="N335" s="92"/>
+      <c r="O335" s="92"/>
+      <c r="P335" s="92"/>
+      <c r="Q335" s="92"/>
+      <c r="R335" s="92"/>
+      <c r="S335" s="92"/>
+      <c r="T335" s="92"/>
+      <c r="U335" s="92"/>
+      <c r="V335" s="92"/>
+      <c r="W335" s="92"/>
+      <c r="X335" s="92"/>
+      <c r="Y335" s="92"/>
+      <c r="Z335" s="92"/>
+    </row>
+    <row r="336" spans="1:26" ht="13">
+      <c r="A336" s="92" t="s">
+        <v>41</v>
+      </c>
+      <c r="B336" s="92" t="s">
+        <v>850</v>
+      </c>
+      <c r="C336" s="92"/>
+      <c r="D336" s="92"/>
+      <c r="E336" s="92"/>
+      <c r="F336" s="92"/>
+      <c r="G336" s="92"/>
+      <c r="H336" s="92"/>
+      <c r="I336" s="92"/>
+      <c r="J336" s="92"/>
+      <c r="K336" s="92"/>
+      <c r="L336" s="92" t="s">
+        <v>851</v>
+      </c>
+      <c r="M336" s="92"/>
+      <c r="N336" s="92"/>
+      <c r="O336" s="92"/>
+      <c r="P336" s="92"/>
+      <c r="Q336" s="92"/>
+      <c r="R336" s="92"/>
+      <c r="S336" s="92"/>
+      <c r="T336" s="92"/>
+      <c r="U336" s="92"/>
+      <c r="V336" s="92"/>
+      <c r="W336" s="92"/>
+      <c r="X336" s="92"/>
+      <c r="Y336" s="92"/>
+      <c r="Z336" s="92"/>
+    </row>
+    <row r="337" spans="1:26" ht="13">
+      <c r="A337" s="92" t="s">
+        <v>41</v>
+      </c>
+      <c r="B337" s="92" t="s">
+        <v>852</v>
+      </c>
+      <c r="C337" s="92"/>
+      <c r="D337" s="92"/>
+      <c r="E337" s="92"/>
+      <c r="F337" s="92"/>
+      <c r="G337" s="92"/>
+      <c r="H337" s="92"/>
+      <c r="I337" s="92"/>
+      <c r="J337" s="92"/>
+      <c r="K337" s="92"/>
+      <c r="L337" s="92" t="s">
+        <v>853</v>
+      </c>
+      <c r="M337" s="92"/>
+      <c r="N337" s="92"/>
+      <c r="O337" s="92"/>
+      <c r="P337" s="92"/>
+      <c r="Q337" s="92"/>
+      <c r="R337" s="92"/>
+      <c r="S337" s="92"/>
+      <c r="T337" s="92"/>
+      <c r="U337" s="92"/>
+      <c r="V337" s="92"/>
+      <c r="W337" s="92"/>
+      <c r="X337" s="92"/>
+      <c r="Y337" s="92"/>
+      <c r="Z337" s="92"/>
+    </row>
+    <row r="338" spans="1:26" ht="13">
+      <c r="A338" s="2"/>
+      <c r="L338" s="2"/>
+    </row>
+    <row r="339" spans="1:26" ht="13">
+      <c r="A339" s="2"/>
+      <c r="L339" s="2"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -21292,7 +21444,7 @@
       </c>
     </row>
     <row r="212" spans="1:4" ht="13">
-      <c r="A212" s="7" t="s">
+      <c r="A212" s="46" t="s">
         <v>281</v>
       </c>
       <c r="B212" s="2" t="s">

</xml_diff>

<commit_message>
Added relevancy condition to hide the local herbs explanation if it has already occured earlier
</commit_message>
<xml_diff>
--- a/forms/app/pregnancy.xlsx
+++ b/forms/app/pregnancy.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2477" uniqueCount="1432">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2478" uniqueCount="1433">
   <si>
     <t>type</t>
   </si>
@@ -4503,6 +4503,9 @@
   </si>
   <si>
     <t>selected(${delivery_complications},'big_baby') or selected(${big_baby},"yes")</t>
+  </si>
+  <si>
+    <t>selected(${local_herbs},'no')</t>
   </si>
 </sst>
 </file>
@@ -14011,7 +14014,9 @@
         <v>301</v>
       </c>
       <c r="E246" s="56"/>
-      <c r="F246" s="56"/>
+      <c r="F246" s="69" t="s">
+        <v>1432</v>
+      </c>
       <c r="G246" s="56"/>
       <c r="H246" s="56"/>
       <c r="I246" s="56"/>
@@ -21767,6 +21772,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
solved missing shehia bug
</commit_message>
<xml_diff>
--- a/forms/app/pregnancy.xlsx
+++ b/forms/app/pregnancy.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2481" uniqueCount="1435">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2482" uniqueCount="1437">
   <si>
     <t xml:space="preserve">type</t>
   </si>
@@ -2737,6 +2737,32 @@
 </t>
   </si>
   <si>
+    <t xml:space="preserve">${enabel} = "true" and (
+  selected(${previous_delivery_by_c_section},"yes") or selected(${previous_delivery_by_vacuum},"yes")
+  or selected(${previous_stillbirth},"yes")
+  or selected(${delivery_complications},'prolonged_labor')
+  or selected(${delivery_complications},'large_perineal_tear')
+  or selected(${delivery_complications},'retained_placenta')
+  or selected(${delivery_complications},'aph')
+  or selected(${delivery_complications},'postpartum_hemorrage')
+  or selected(${delivery_complications},'eclampsia')
+  or selected(${delivery_complications},'big_baby') or selected(${big_baby},"yes")
+  or ${previous_miscarriages} &gt; 0 and ${enabel}=”true”
+  or selected(${multiple_pregnancy},"yes")
+  or selected(${malpresentation},"yes")
+  or selected(${breech_position},"yes")
+  or selected(${medical_conditions},"high_blood_pressure")
+  or selected(${medical_conditions},"diabetes")
+  or selected(${medical_conditions},"sickle_cell")
+  or selected(${medical_conditions},"cardiac_disease")
+  or selected(${higher_facility_delivery},"yes")
+  or selected(${allow_partner_to_deliver_facility},"no") or selected(${partner_not_present},"yes") 
+  or selected(${ten_or_more_years},"yes")
+  or selected(${nutrition_restrictions},"yes")
+  or selected(${local_herbs},"yes")
+)</t>
+  </si>
+  <si>
     <t xml:space="preserve">c_section_risk</t>
   </si>
   <si>
@@ -2866,6 +2892,9 @@
   </si>
   <si>
     <t xml:space="preserve">Mimba kuharibika </t>
+  </si>
+  <si>
+    <t xml:space="preserve">${previous_miscarriages} &gt; 0 and ${enabel}=”true”</t>
   </si>
   <si>
     <t xml:space="preserve">multiple_pregnancy_risk</t>
@@ -15601,7 +15630,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="303" customFormat="false" ht="39" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="303" customFormat="false" ht="280.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A303" s="2" t="s">
         <v>109</v>
       </c>
@@ -15614,7 +15643,9 @@
       <c r="D303" s="12" t="s">
         <v>845</v>
       </c>
-      <c r="F303" s="2"/>
+      <c r="F303" s="12" t="s">
+        <v>846</v>
+      </c>
       <c r="G303" s="2"/>
     </row>
     <row r="304" customFormat="false" ht="13" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15622,16 +15653,16 @@
         <v>109</v>
       </c>
       <c r="B304" s="2" t="s">
-        <v>846</v>
+        <v>847</v>
       </c>
       <c r="C304" s="12" t="s">
-        <v>847</v>
+        <v>848</v>
       </c>
       <c r="D304" s="2" t="s">
-        <v>848</v>
+        <v>849</v>
       </c>
       <c r="F304" s="2" t="s">
-        <v>849</v>
+        <v>850</v>
       </c>
       <c r="G304" s="2"/>
     </row>
@@ -15640,16 +15671,16 @@
         <v>109</v>
       </c>
       <c r="B305" s="2" t="s">
-        <v>850</v>
+        <v>851</v>
       </c>
       <c r="C305" s="12" t="s">
-        <v>851</v>
+        <v>852</v>
       </c>
       <c r="D305" s="4" t="s">
-        <v>852</v>
+        <v>853</v>
       </c>
       <c r="F305" s="2" t="s">
-        <v>853</v>
+        <v>854</v>
       </c>
       <c r="G305" s="2"/>
     </row>
@@ -15658,16 +15689,16 @@
         <v>109</v>
       </c>
       <c r="B306" s="2" t="s">
-        <v>854</v>
+        <v>855</v>
       </c>
       <c r="C306" s="12" t="s">
-        <v>855</v>
+        <v>856</v>
       </c>
       <c r="D306" s="4" t="s">
-        <v>856</v>
+        <v>857</v>
       </c>
       <c r="F306" s="2" t="s">
-        <v>857</v>
+        <v>858</v>
       </c>
       <c r="G306" s="2"/>
     </row>
@@ -15676,16 +15707,16 @@
         <v>109</v>
       </c>
       <c r="B307" s="2" t="s">
-        <v>858</v>
+        <v>859</v>
       </c>
       <c r="C307" s="2" t="s">
-        <v>859</v>
+        <v>860</v>
       </c>
       <c r="D307" s="2" t="s">
-        <v>860</v>
+        <v>861</v>
       </c>
       <c r="F307" s="12" t="s">
-        <v>861</v>
+        <v>862</v>
       </c>
       <c r="G307" s="2"/>
       <c r="L307" s="4"/>
@@ -15695,16 +15726,16 @@
         <v>109</v>
       </c>
       <c r="B308" s="2" t="s">
-        <v>862</v>
+        <v>863</v>
       </c>
       <c r="C308" s="12" t="s">
-        <v>863</v>
+        <v>864</v>
       </c>
       <c r="D308" s="2" t="s">
-        <v>864</v>
+        <v>865</v>
       </c>
       <c r="F308" s="12" t="s">
-        <v>865</v>
+        <v>866</v>
       </c>
       <c r="G308" s="2"/>
       <c r="L308" s="4"/>
@@ -15714,16 +15745,16 @@
         <v>109</v>
       </c>
       <c r="B309" s="2" t="s">
-        <v>866</v>
+        <v>867</v>
       </c>
       <c r="C309" s="12" t="s">
-        <v>867</v>
+        <v>868</v>
       </c>
       <c r="D309" s="2" t="s">
-        <v>868</v>
+        <v>869</v>
       </c>
       <c r="F309" s="12" t="s">
-        <v>869</v>
+        <v>870</v>
       </c>
       <c r="G309" s="2"/>
       <c r="L309" s="4"/>
@@ -15733,16 +15764,16 @@
         <v>109</v>
       </c>
       <c r="B310" s="2" t="s">
-        <v>870</v>
+        <v>871</v>
       </c>
       <c r="C310" s="12" t="s">
-        <v>871</v>
+        <v>872</v>
       </c>
       <c r="D310" s="2" t="s">
-        <v>872</v>
+        <v>873</v>
       </c>
       <c r="F310" s="12" t="s">
-        <v>873</v>
+        <v>874</v>
       </c>
       <c r="G310" s="2"/>
       <c r="L310" s="4"/>
@@ -15752,16 +15783,16 @@
         <v>109</v>
       </c>
       <c r="B311" s="2" t="s">
-        <v>874</v>
+        <v>875</v>
       </c>
       <c r="C311" s="12" t="s">
-        <v>875</v>
+        <v>876</v>
       </c>
       <c r="D311" s="2" t="s">
-        <v>876</v>
+        <v>877</v>
       </c>
       <c r="F311" s="12" t="s">
-        <v>877</v>
+        <v>878</v>
       </c>
       <c r="G311" s="2"/>
       <c r="L311" s="4"/>
@@ -15771,16 +15802,16 @@
         <v>109</v>
       </c>
       <c r="B312" s="2" t="s">
-        <v>878</v>
+        <v>879</v>
       </c>
       <c r="C312" s="2" t="s">
-        <v>879</v>
+        <v>880</v>
       </c>
       <c r="D312" s="2" t="s">
         <v>457</v>
       </c>
       <c r="F312" s="12" t="s">
-        <v>880</v>
+        <v>881</v>
       </c>
       <c r="G312" s="2"/>
       <c r="L312" s="4"/>
@@ -15790,35 +15821,35 @@
         <v>109</v>
       </c>
       <c r="B313" s="2" t="s">
-        <v>881</v>
+        <v>882</v>
       </c>
       <c r="C313" s="12" t="s">
-        <v>882</v>
+        <v>883</v>
       </c>
       <c r="D313" s="2" t="s">
-        <v>883</v>
+        <v>884</v>
       </c>
       <c r="F313" s="12" t="s">
-        <v>884</v>
+        <v>885</v>
       </c>
       <c r="G313" s="2"/>
       <c r="L313" s="4"/>
     </row>
-    <row r="314" s="36" customFormat="true" ht="13" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="314" s="36" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A314" s="2" t="s">
         <v>109</v>
       </c>
       <c r="B314" s="2" t="s">
-        <v>885</v>
+        <v>886</v>
       </c>
       <c r="C314" s="12" t="s">
-        <v>886</v>
+        <v>887</v>
       </c>
       <c r="D314" s="4" t="s">
-        <v>887</v>
+        <v>888</v>
       </c>
       <c r="F314" s="2" t="s">
-        <v>257</v>
+        <v>889</v>
       </c>
       <c r="G314" s="2"/>
     </row>
@@ -15827,16 +15858,16 @@
         <v>109</v>
       </c>
       <c r="B315" s="2" t="s">
-        <v>888</v>
+        <v>890</v>
       </c>
       <c r="C315" s="12" t="s">
-        <v>889</v>
+        <v>891</v>
       </c>
       <c r="D315" s="4" t="s">
-        <v>890</v>
+        <v>892</v>
       </c>
       <c r="F315" s="2" t="s">
-        <v>891</v>
+        <v>893</v>
       </c>
       <c r="G315" s="2"/>
     </row>
@@ -15845,16 +15876,16 @@
         <v>109</v>
       </c>
       <c r="B316" s="2" t="s">
-        <v>892</v>
+        <v>894</v>
       </c>
       <c r="C316" s="12" t="s">
-        <v>893</v>
+        <v>895</v>
       </c>
       <c r="D316" s="4" t="s">
-        <v>894</v>
+        <v>896</v>
       </c>
       <c r="F316" s="2" t="s">
-        <v>895</v>
+        <v>897</v>
       </c>
       <c r="G316" s="2"/>
     </row>
@@ -15863,16 +15894,16 @@
         <v>109</v>
       </c>
       <c r="B317" s="12" t="s">
-        <v>896</v>
+        <v>898</v>
       </c>
       <c r="C317" s="12" t="s">
-        <v>897</v>
+        <v>899</v>
       </c>
       <c r="D317" s="4" t="s">
-        <v>898</v>
+        <v>900</v>
       </c>
       <c r="F317" s="2" t="s">
-        <v>899</v>
+        <v>901</v>
       </c>
       <c r="G317" s="2"/>
     </row>
@@ -15881,16 +15912,16 @@
         <v>109</v>
       </c>
       <c r="B318" s="2" t="s">
-        <v>900</v>
+        <v>902</v>
       </c>
       <c r="C318" s="2" t="s">
-        <v>901</v>
+        <v>903</v>
       </c>
       <c r="D318" s="2" t="s">
-        <v>902</v>
+        <v>904</v>
       </c>
       <c r="F318" s="2" t="s">
-        <v>903</v>
+        <v>905</v>
       </c>
       <c r="G318" s="2"/>
     </row>
@@ -15899,16 +15930,16 @@
         <v>109</v>
       </c>
       <c r="B319" s="2" t="s">
-        <v>904</v>
+        <v>906</v>
       </c>
       <c r="C319" s="2" t="s">
-        <v>905</v>
+        <v>907</v>
       </c>
       <c r="D319" s="2" t="s">
-        <v>906</v>
+        <v>908</v>
       </c>
       <c r="F319" s="2" t="s">
-        <v>907</v>
+        <v>909</v>
       </c>
       <c r="G319" s="2"/>
     </row>
@@ -15917,16 +15948,16 @@
         <v>109</v>
       </c>
       <c r="B320" s="2" t="s">
-        <v>908</v>
+        <v>910</v>
       </c>
       <c r="C320" s="12" t="s">
-        <v>909</v>
+        <v>911</v>
       </c>
       <c r="D320" s="2" t="s">
-        <v>910</v>
+        <v>912</v>
       </c>
       <c r="F320" s="2" t="s">
-        <v>911</v>
+        <v>913</v>
       </c>
       <c r="G320" s="2"/>
     </row>
@@ -15935,16 +15966,16 @@
         <v>109</v>
       </c>
       <c r="B321" s="2" t="s">
-        <v>912</v>
+        <v>914</v>
       </c>
       <c r="C321" s="2" t="s">
-        <v>913</v>
+        <v>915</v>
       </c>
       <c r="D321" s="2" t="s">
-        <v>914</v>
+        <v>916</v>
       </c>
       <c r="F321" s="2" t="s">
-        <v>915</v>
+        <v>917</v>
       </c>
       <c r="G321" s="2"/>
     </row>
@@ -15953,16 +15984,16 @@
         <v>109</v>
       </c>
       <c r="B322" s="2" t="s">
-        <v>916</v>
+        <v>918</v>
       </c>
       <c r="C322" s="12" t="s">
-        <v>917</v>
+        <v>919</v>
       </c>
       <c r="D322" s="4" t="s">
-        <v>918</v>
+        <v>920</v>
       </c>
       <c r="F322" s="2" t="s">
-        <v>919</v>
+        <v>921</v>
       </c>
       <c r="G322" s="2"/>
     </row>
@@ -15971,16 +16002,16 @@
         <v>109</v>
       </c>
       <c r="B323" s="2" t="s">
-        <v>920</v>
+        <v>922</v>
       </c>
       <c r="C323" s="12" t="s">
-        <v>921</v>
+        <v>923</v>
       </c>
       <c r="D323" s="4" t="s">
-        <v>922</v>
+        <v>924</v>
       </c>
       <c r="F323" s="2" t="s">
-        <v>923</v>
+        <v>925</v>
       </c>
       <c r="G323" s="2"/>
     </row>
@@ -15989,16 +16020,16 @@
         <v>109</v>
       </c>
       <c r="B324" s="2" t="s">
-        <v>924</v>
+        <v>926</v>
       </c>
       <c r="C324" s="12" t="s">
-        <v>925</v>
+        <v>927</v>
       </c>
       <c r="D324" s="4" t="s">
-        <v>926</v>
+        <v>928</v>
       </c>
       <c r="F324" s="2" t="s">
-        <v>927</v>
+        <v>929</v>
       </c>
       <c r="G324" s="2"/>
     </row>
@@ -16007,16 +16038,16 @@
         <v>109</v>
       </c>
       <c r="B325" s="2" t="s">
-        <v>928</v>
+        <v>930</v>
       </c>
       <c r="C325" s="12" t="s">
-        <v>929</v>
+        <v>931</v>
       </c>
       <c r="D325" s="4" t="s">
-        <v>930</v>
+        <v>932</v>
       </c>
       <c r="F325" s="2" t="s">
-        <v>931</v>
+        <v>933</v>
       </c>
       <c r="G325" s="2"/>
     </row>
@@ -16025,16 +16056,16 @@
         <v>109</v>
       </c>
       <c r="B326" s="2" t="s">
-        <v>932</v>
+        <v>934</v>
       </c>
       <c r="C326" s="12" t="s">
-        <v>933</v>
+        <v>935</v>
       </c>
       <c r="D326" s="4" t="s">
-        <v>934</v>
+        <v>936</v>
       </c>
       <c r="F326" s="2" t="s">
-        <v>935</v>
+        <v>937</v>
       </c>
       <c r="G326" s="2"/>
     </row>
@@ -16043,17 +16074,17 @@
         <v>109</v>
       </c>
       <c r="B327" s="37" t="s">
-        <v>936</v>
+        <v>938</v>
       </c>
       <c r="C327" s="37" t="s">
-        <v>937</v>
+        <v>939</v>
       </c>
       <c r="D327" s="38" t="s">
-        <v>938</v>
+        <v>940</v>
       </c>
       <c r="E327" s="37"/>
       <c r="F327" s="38" t="s">
-        <v>939</v>
+        <v>941</v>
       </c>
       <c r="G327" s="37"/>
       <c r="H327" s="37"/>
@@ -16081,17 +16112,17 @@
         <v>109</v>
       </c>
       <c r="B328" s="37" t="s">
-        <v>940</v>
+        <v>942</v>
       </c>
       <c r="C328" s="37" t="s">
-        <v>941</v>
+        <v>943</v>
       </c>
       <c r="D328" s="38" t="s">
-        <v>942</v>
+        <v>944</v>
       </c>
       <c r="E328" s="37"/>
       <c r="F328" s="37" t="s">
-        <v>943</v>
+        <v>945</v>
       </c>
       <c r="G328" s="37"/>
       <c r="H328" s="37"/>
@@ -16119,20 +16150,20 @@
         <v>109</v>
       </c>
       <c r="B329" s="37" t="s">
-        <v>944</v>
+        <v>946</v>
       </c>
       <c r="C329" s="37" t="s">
-        <v>945</v>
+        <v>947</v>
       </c>
       <c r="D329" s="39" t="s">
-        <v>946</v>
+        <v>948</v>
       </c>
       <c r="E329" s="37"/>
       <c r="F329" s="40" t="s">
-        <v>947</v>
+        <v>949</v>
       </c>
       <c r="G329" s="37" t="s">
-        <v>948</v>
+        <v>950</v>
       </c>
       <c r="H329" s="37"/>
       <c r="I329" s="37"/>
@@ -16159,20 +16190,20 @@
         <v>109</v>
       </c>
       <c r="B330" s="37" t="s">
-        <v>949</v>
+        <v>951</v>
       </c>
       <c r="C330" s="37" t="s">
-        <v>950</v>
+        <v>952</v>
       </c>
       <c r="D330" s="37" t="s">
-        <v>951</v>
+        <v>953</v>
       </c>
       <c r="E330" s="37"/>
       <c r="F330" s="41" t="s">
-        <v>952</v>
+        <v>954</v>
       </c>
       <c r="G330" s="37" t="s">
-        <v>948</v>
+        <v>950</v>
       </c>
       <c r="H330" s="37"/>
       <c r="I330" s="37"/>
@@ -16199,20 +16230,20 @@
         <v>109</v>
       </c>
       <c r="B331" s="37" t="s">
-        <v>953</v>
+        <v>955</v>
       </c>
       <c r="C331" s="37" t="s">
-        <v>954</v>
+        <v>956</v>
       </c>
       <c r="D331" s="38" t="s">
-        <v>955</v>
+        <v>957</v>
       </c>
       <c r="E331" s="37"/>
       <c r="F331" s="37" t="s">
-        <v>956</v>
+        <v>958</v>
       </c>
       <c r="G331" s="37" t="s">
-        <v>948</v>
+        <v>950</v>
       </c>
       <c r="H331" s="37"/>
       <c r="I331" s="37"/>
@@ -16251,7 +16282,7 @@
         <v>41</v>
       </c>
       <c r="B333" s="37" t="s">
-        <v>957</v>
+        <v>959</v>
       </c>
       <c r="C333" s="37"/>
       <c r="D333" s="37"/>
@@ -16263,7 +16294,7 @@
       <c r="J333" s="37"/>
       <c r="K333" s="37"/>
       <c r="L333" s="37" t="s">
-        <v>958</v>
+        <v>960</v>
       </c>
       <c r="M333" s="37"/>
       <c r="N333" s="37"/>
@@ -16285,7 +16316,7 @@
         <v>41</v>
       </c>
       <c r="B334" s="37" t="s">
-        <v>959</v>
+        <v>961</v>
       </c>
       <c r="C334" s="37"/>
       <c r="D334" s="37"/>
@@ -16297,7 +16328,7 @@
       <c r="J334" s="37"/>
       <c r="K334" s="37"/>
       <c r="L334" s="37" t="s">
-        <v>960</v>
+        <v>962</v>
       </c>
       <c r="M334" s="37"/>
       <c r="N334" s="37"/>
@@ -16319,7 +16350,7 @@
         <v>41</v>
       </c>
       <c r="B335" s="37" t="s">
-        <v>961</v>
+        <v>963</v>
       </c>
       <c r="C335" s="37"/>
       <c r="D335" s="37"/>
@@ -16331,7 +16362,7 @@
       <c r="J335" s="37"/>
       <c r="K335" s="37"/>
       <c r="L335" s="37" t="s">
-        <v>962</v>
+        <v>964</v>
       </c>
       <c r="M335" s="37"/>
       <c r="N335" s="37"/>
@@ -16353,7 +16384,7 @@
         <v>41</v>
       </c>
       <c r="B336" s="37" t="s">
-        <v>963</v>
+        <v>965</v>
       </c>
       <c r="C336" s="37"/>
       <c r="D336" s="37"/>
@@ -16365,7 +16396,7 @@
       <c r="J336" s="37"/>
       <c r="K336" s="37"/>
       <c r="L336" s="37" t="s">
-        <v>964</v>
+        <v>966</v>
       </c>
       <c r="M336" s="37"/>
       <c r="N336" s="37"/>
@@ -16387,7 +16418,7 @@
         <v>41</v>
       </c>
       <c r="B337" s="37" t="s">
-        <v>965</v>
+        <v>967</v>
       </c>
       <c r="C337" s="37"/>
       <c r="D337" s="37"/>
@@ -16399,7 +16430,7 @@
       <c r="J337" s="37"/>
       <c r="K337" s="37"/>
       <c r="L337" s="37" t="s">
-        <v>966</v>
+        <v>968</v>
       </c>
       <c r="M337" s="37"/>
       <c r="N337" s="37"/>
@@ -16455,7 +16486,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="42" t="s">
-        <v>967</v>
+        <v>969</v>
       </c>
       <c r="B1" s="42" t="s">
         <v>1</v>
@@ -16472,30 +16503,30 @@
     </row>
     <row r="2" customFormat="false" ht="14.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="43" t="s">
-        <v>968</v>
+        <v>970</v>
       </c>
       <c r="B2" s="43" t="s">
         <v>139</v>
       </c>
       <c r="C2" s="43" t="s">
-        <v>969</v>
+        <v>971</v>
       </c>
       <c r="D2" s="43" t="s">
-        <v>970</v>
+        <v>972</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="14.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="43" t="s">
-        <v>968</v>
+        <v>970</v>
       </c>
       <c r="B3" s="43" t="s">
-        <v>971</v>
+        <v>973</v>
       </c>
       <c r="C3" s="43" t="s">
-        <v>972</v>
+        <v>974</v>
       </c>
       <c r="D3" s="43" t="s">
-        <v>973</v>
+        <v>975</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -16503,13 +16534,13 @@
         <v>474</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>974</v>
+        <v>976</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>975</v>
+        <v>977</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>976</v>
+        <v>978</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -16517,13 +16548,13 @@
         <v>474</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>977</v>
+        <v>979</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>978</v>
+        <v>980</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>979</v>
+        <v>981</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -16531,13 +16562,13 @@
         <v>474</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>980</v>
+        <v>982</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>981</v>
+        <v>983</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>982</v>
+        <v>984</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -16545,13 +16576,13 @@
         <v>474</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>983</v>
+        <v>985</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>984</v>
+        <v>986</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>985</v>
+        <v>987</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -16559,13 +16590,13 @@
         <v>474</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>986</v>
+        <v>988</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>987</v>
+        <v>989</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>988</v>
+        <v>990</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -16573,13 +16604,13 @@
         <v>474</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>989</v>
+        <v>991</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>990</v>
+        <v>992</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>991</v>
+        <v>993</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -16587,13 +16618,13 @@
         <v>474</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>992</v>
+        <v>994</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>993</v>
+        <v>995</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>994</v>
+        <v>996</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -16601,13 +16632,13 @@
         <v>474</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>995</v>
+        <v>997</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>996</v>
+        <v>998</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>997</v>
+        <v>999</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -16615,13 +16646,13 @@
         <v>474</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>998</v>
+        <v>1000</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>999</v>
+        <v>1001</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>1000</v>
+        <v>1002</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -16629,13 +16660,13 @@
         <v>474</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>1001</v>
+        <v>1003</v>
       </c>
       <c r="C13" s="14" t="s">
-        <v>1002</v>
+        <v>1004</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>1003</v>
+        <v>1005</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -16643,13 +16674,13 @@
         <v>474</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>1004</v>
+        <v>1006</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>1005</v>
+        <v>1007</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>1006</v>
+        <v>1008</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -16657,13 +16688,13 @@
         <v>474</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>1007</v>
+        <v>1009</v>
       </c>
       <c r="C15" s="14" t="s">
-        <v>1008</v>
+        <v>1010</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>1009</v>
+        <v>1011</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -16671,13 +16702,13 @@
         <v>474</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>1010</v>
+        <v>1012</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>1011</v>
+        <v>1013</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>1012</v>
+        <v>1014</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -16685,13 +16716,13 @@
         <v>474</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>1013</v>
+        <v>1015</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>1014</v>
+        <v>1016</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>1015</v>
+        <v>1017</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="13" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16699,13 +16730,13 @@
         <v>538</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>1016</v>
+        <v>1018</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>1017</v>
+        <v>1019</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>1018</v>
+        <v>1020</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="13" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16713,13 +16744,13 @@
         <v>538</v>
       </c>
       <c r="B19" s="4" t="s">
-        <v>1019</v>
+        <v>1021</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>1020</v>
+        <v>1022</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>1021</v>
+        <v>1023</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="13" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16727,13 +16758,13 @@
         <v>569</v>
       </c>
       <c r="B20" s="4" t="s">
-        <v>1022</v>
+        <v>1024</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>1023</v>
+        <v>1025</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>1024</v>
+        <v>1026</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="13" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16741,13 +16772,13 @@
         <v>569</v>
       </c>
       <c r="B21" s="4" t="s">
-        <v>1025</v>
+        <v>1027</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>1026</v>
+        <v>1028</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>1027</v>
+        <v>1029</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="13" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16755,13 +16786,13 @@
         <v>569</v>
       </c>
       <c r="B22" s="4" t="s">
-        <v>1028</v>
+        <v>1030</v>
       </c>
       <c r="C22" s="4" t="s">
-        <v>1029</v>
+        <v>1031</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>1030</v>
+        <v>1032</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="13" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16769,13 +16800,13 @@
         <v>569</v>
       </c>
       <c r="B23" s="4" t="s">
-        <v>1031</v>
+        <v>1033</v>
       </c>
       <c r="C23" s="4" t="s">
-        <v>1032</v>
+        <v>1034</v>
       </c>
       <c r="D23" s="2" t="s">
-        <v>1033</v>
+        <v>1035</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="13" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16783,13 +16814,13 @@
         <v>569</v>
       </c>
       <c r="B24" s="4" t="s">
-        <v>1034</v>
+        <v>1036</v>
       </c>
       <c r="C24" s="4" t="s">
-        <v>1035</v>
+        <v>1037</v>
       </c>
       <c r="D24" s="2" t="s">
-        <v>1036</v>
+        <v>1038</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="13" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16797,13 +16828,13 @@
         <v>569</v>
       </c>
       <c r="B25" s="4" t="s">
-        <v>1037</v>
+        <v>1039</v>
       </c>
       <c r="C25" s="4" t="s">
-        <v>1038</v>
+        <v>1040</v>
       </c>
       <c r="D25" s="2" t="s">
-        <v>1039</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="13" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16811,13 +16842,13 @@
         <v>569</v>
       </c>
       <c r="B26" s="4" t="s">
-        <v>1040</v>
+        <v>1042</v>
       </c>
       <c r="C26" s="4" t="s">
-        <v>1041</v>
+        <v>1043</v>
       </c>
       <c r="D26" s="2" t="s">
-        <v>1042</v>
+        <v>1044</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="13" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16825,13 +16856,13 @@
         <v>589</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>1043</v>
+        <v>1045</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>1044</v>
+        <v>1046</v>
       </c>
       <c r="D27" s="2" t="s">
-        <v>1045</v>
+        <v>1047</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="13" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16839,13 +16870,13 @@
         <v>589</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>1046</v>
+        <v>1048</v>
       </c>
       <c r="C28" s="5" t="s">
-        <v>1047</v>
+        <v>1049</v>
       </c>
       <c r="D28" s="5" t="s">
-        <v>1048</v>
+        <v>1050</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="13" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16853,13 +16884,13 @@
         <v>589</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>1049</v>
+        <v>1051</v>
       </c>
       <c r="C29" s="5" t="s">
-        <v>1050</v>
+        <v>1052</v>
       </c>
       <c r="D29" s="2" t="s">
-        <v>1051</v>
+        <v>1053</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="13" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16867,13 +16898,13 @@
         <v>589</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>1052</v>
+        <v>1054</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>1053</v>
+        <v>1055</v>
       </c>
       <c r="D30" s="2" t="s">
-        <v>1054</v>
+        <v>1056</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="13" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16881,13 +16912,13 @@
         <v>589</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>1055</v>
+        <v>1057</v>
       </c>
       <c r="C31" s="5" t="s">
-        <v>1056</v>
+        <v>1058</v>
       </c>
       <c r="D31" s="5" t="s">
-        <v>1057</v>
+        <v>1059</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="13" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16895,13 +16926,13 @@
         <v>589</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>1058</v>
+        <v>1060</v>
       </c>
       <c r="C32" s="5" t="s">
-        <v>1059</v>
+        <v>1061</v>
       </c>
       <c r="D32" s="2" t="s">
-        <v>1060</v>
+        <v>1062</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="13" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16909,13 +16940,13 @@
         <v>589</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>1061</v>
+        <v>1063</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>1062</v>
+        <v>1064</v>
       </c>
       <c r="D33" s="2" t="s">
-        <v>1063</v>
+        <v>1065</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="13" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16923,13 +16954,13 @@
         <v>589</v>
       </c>
       <c r="B34" s="4" t="s">
-        <v>1064</v>
+        <v>1066</v>
       </c>
       <c r="C34" s="4" t="s">
-        <v>1065</v>
+        <v>1067</v>
       </c>
       <c r="D34" s="2" t="s">
-        <v>1066</v>
+        <v>1068</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="13" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16937,13 +16968,13 @@
         <v>313</v>
       </c>
       <c r="B35" s="4" t="s">
-        <v>1067</v>
+        <v>1069</v>
       </c>
       <c r="C35" s="4" t="s">
-        <v>1068</v>
+        <v>1070</v>
       </c>
       <c r="D35" s="2" t="s">
-        <v>1069</v>
+        <v>1071</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="13" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16951,13 +16982,13 @@
         <v>313</v>
       </c>
       <c r="B36" s="4" t="s">
-        <v>1070</v>
+        <v>1072</v>
       </c>
       <c r="C36" s="4" t="s">
-        <v>1071</v>
+        <v>1073</v>
       </c>
       <c r="D36" s="2" t="s">
-        <v>1072</v>
+        <v>1074</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="13" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16965,13 +16996,13 @@
         <v>313</v>
       </c>
       <c r="B37" s="4" t="s">
-        <v>1073</v>
+        <v>1075</v>
       </c>
       <c r="C37" s="4" t="s">
-        <v>1074</v>
+        <v>1076</v>
       </c>
       <c r="D37" s="2" t="s">
-        <v>1075</v>
+        <v>1077</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="13" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16979,13 +17010,13 @@
         <v>721</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>1076</v>
+        <v>1078</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>1077</v>
+        <v>1079</v>
       </c>
       <c r="D38" s="2" t="s">
-        <v>1077</v>
+        <v>1079</v>
       </c>
       <c r="E38" s="2"/>
       <c r="F38" s="2"/>
@@ -17015,13 +17046,13 @@
         <v>721</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>1078</v>
+        <v>1080</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>1079</v>
+        <v>1081</v>
       </c>
       <c r="D39" s="2" t="s">
-        <v>1079</v>
+        <v>1081</v>
       </c>
       <c r="E39" s="2"/>
       <c r="F39" s="2"/>
@@ -17051,13 +17082,13 @@
         <v>721</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>1080</v>
+        <v>1082</v>
       </c>
       <c r="C40" s="2" t="s">
-        <v>1081</v>
+        <v>1083</v>
       </c>
       <c r="D40" s="2" t="s">
-        <v>1082</v>
+        <v>1084</v>
       </c>
       <c r="E40" s="2"/>
       <c r="F40" s="2"/>
@@ -17087,16 +17118,16 @@
         <v>726</v>
       </c>
       <c r="B41" s="2" t="s">
-        <v>1083</v>
+        <v>1085</v>
       </c>
       <c r="C41" s="2" t="s">
-        <v>1084</v>
+        <v>1086</v>
       </c>
       <c r="D41" s="2" t="s">
-        <v>1084</v>
+        <v>1086</v>
       </c>
       <c r="E41" s="2" t="s">
-        <v>1076</v>
+        <v>1078</v>
       </c>
       <c r="F41" s="2"/>
       <c r="G41" s="2"/>
@@ -17125,16 +17156,16 @@
         <v>726</v>
       </c>
       <c r="B42" s="2" t="s">
-        <v>1085</v>
+        <v>1087</v>
       </c>
       <c r="C42" s="2" t="s">
-        <v>1086</v>
+        <v>1088</v>
       </c>
       <c r="D42" s="2" t="s">
-        <v>1086</v>
+        <v>1088</v>
       </c>
       <c r="E42" s="2" t="s">
-        <v>1076</v>
+        <v>1078</v>
       </c>
       <c r="F42" s="2"/>
       <c r="G42" s="2"/>
@@ -17163,16 +17194,16 @@
         <v>726</v>
       </c>
       <c r="B43" s="2" t="s">
-        <v>1087</v>
+        <v>1089</v>
       </c>
       <c r="C43" s="2" t="s">
-        <v>1088</v>
+        <v>1090</v>
       </c>
       <c r="D43" s="2" t="s">
-        <v>1088</v>
+        <v>1090</v>
       </c>
       <c r="E43" s="2" t="s">
-        <v>1076</v>
+        <v>1078</v>
       </c>
       <c r="F43" s="2"/>
       <c r="G43" s="2"/>
@@ -17201,16 +17232,16 @@
         <v>726</v>
       </c>
       <c r="B44" s="2" t="s">
-        <v>1089</v>
+        <v>1091</v>
       </c>
       <c r="C44" s="2" t="s">
-        <v>1090</v>
+        <v>1092</v>
       </c>
       <c r="D44" s="2" t="s">
-        <v>1090</v>
+        <v>1092</v>
       </c>
       <c r="E44" s="2" t="s">
-        <v>1076</v>
+        <v>1078</v>
       </c>
       <c r="F44" s="2"/>
       <c r="G44" s="2"/>
@@ -17239,16 +17270,16 @@
         <v>726</v>
       </c>
       <c r="B45" s="2" t="s">
-        <v>1091</v>
+        <v>1093</v>
       </c>
       <c r="C45" s="2" t="s">
-        <v>1092</v>
+        <v>1094</v>
       </c>
       <c r="D45" s="2" t="s">
-        <v>1092</v>
+        <v>1094</v>
       </c>
       <c r="E45" s="2" t="s">
-        <v>1076</v>
+        <v>1078</v>
       </c>
       <c r="F45" s="2"/>
       <c r="G45" s="2"/>
@@ -17277,16 +17308,16 @@
         <v>726</v>
       </c>
       <c r="B46" s="2" t="s">
-        <v>1093</v>
+        <v>1095</v>
       </c>
       <c r="C46" s="2" t="s">
-        <v>1094</v>
+        <v>1096</v>
       </c>
       <c r="D46" s="2" t="s">
-        <v>1094</v>
+        <v>1096</v>
       </c>
       <c r="E46" s="2" t="s">
-        <v>1076</v>
+        <v>1078</v>
       </c>
       <c r="F46" s="2"/>
       <c r="G46" s="2"/>
@@ -17315,16 +17346,16 @@
         <v>726</v>
       </c>
       <c r="B47" s="2" t="s">
-        <v>1095</v>
+        <v>1097</v>
       </c>
       <c r="C47" s="2" t="s">
-        <v>1096</v>
+        <v>1098</v>
       </c>
       <c r="D47" s="2" t="s">
-        <v>1096</v>
+        <v>1098</v>
       </c>
       <c r="E47" s="2" t="s">
-        <v>1076</v>
+        <v>1078</v>
       </c>
       <c r="F47" s="2"/>
       <c r="G47" s="2"/>
@@ -17353,16 +17384,16 @@
         <v>726</v>
       </c>
       <c r="B48" s="2" t="s">
-        <v>1097</v>
+        <v>1099</v>
       </c>
       <c r="C48" s="2" t="s">
-        <v>1098</v>
+        <v>1100</v>
       </c>
       <c r="D48" s="2" t="s">
-        <v>1098</v>
+        <v>1100</v>
       </c>
       <c r="E48" s="2" t="s">
-        <v>1078</v>
+        <v>1080</v>
       </c>
       <c r="F48" s="2"/>
       <c r="G48" s="2"/>
@@ -17391,16 +17422,16 @@
         <v>726</v>
       </c>
       <c r="B49" s="2" t="s">
-        <v>1099</v>
+        <v>1101</v>
       </c>
       <c r="C49" s="2" t="s">
-        <v>1100</v>
+        <v>1102</v>
       </c>
       <c r="D49" s="2" t="s">
-        <v>1100</v>
+        <v>1102</v>
       </c>
       <c r="E49" s="2" t="s">
-        <v>1078</v>
+        <v>1080</v>
       </c>
       <c r="F49" s="2"/>
       <c r="G49" s="2"/>
@@ -17429,16 +17460,16 @@
         <v>726</v>
       </c>
       <c r="B50" s="2" t="s">
-        <v>1101</v>
+        <v>1103</v>
       </c>
       <c r="C50" s="2" t="s">
-        <v>1102</v>
+        <v>1104</v>
       </c>
       <c r="D50" s="2" t="s">
-        <v>1102</v>
+        <v>1104</v>
       </c>
       <c r="E50" s="2" t="s">
-        <v>1078</v>
+        <v>1080</v>
       </c>
       <c r="F50" s="2"/>
       <c r="G50" s="2"/>
@@ -17467,16 +17498,16 @@
         <v>726</v>
       </c>
       <c r="B51" s="2" t="s">
-        <v>1103</v>
+        <v>1105</v>
       </c>
       <c r="C51" s="2" t="s">
-        <v>1104</v>
+        <v>1106</v>
       </c>
       <c r="D51" s="2" t="s">
-        <v>1104</v>
+        <v>1106</v>
       </c>
       <c r="E51" s="2" t="s">
-        <v>1078</v>
+        <v>1080</v>
       </c>
       <c r="F51" s="2"/>
       <c r="G51" s="2"/>
@@ -17509,13 +17540,13 @@
         <v>chakechakedistricthospital</v>
       </c>
       <c r="C52" s="5" t="s">
-        <v>1105</v>
+        <v>1107</v>
       </c>
       <c r="D52" s="5" t="s">
-        <v>1106</v>
+        <v>1108</v>
       </c>
       <c r="E52" s="2" t="s">
-        <v>1097</v>
+        <v>1099</v>
       </c>
       <c r="F52" s="2"/>
       <c r="G52" s="2"/>
@@ -17548,13 +17579,13 @@
         <v>pujiniphcu+</v>
       </c>
       <c r="C53" s="2" t="s">
-        <v>1107</v>
+        <v>1109</v>
       </c>
       <c r="D53" s="2" t="s">
-        <v>1107</v>
+        <v>1109</v>
       </c>
       <c r="E53" s="2" t="s">
-        <v>1097</v>
+        <v>1099</v>
       </c>
       <c r="F53" s="2"/>
       <c r="G53" s="2"/>
@@ -17587,13 +17618,13 @@
         <v>tundauwaphcu+</v>
       </c>
       <c r="C54" s="5" t="s">
-        <v>1108</v>
+        <v>1110</v>
       </c>
       <c r="D54" s="5" t="s">
-        <v>1108</v>
+        <v>1110</v>
       </c>
       <c r="E54" s="2" t="s">
-        <v>1097</v>
+        <v>1099</v>
       </c>
       <c r="F54" s="2"/>
       <c r="G54" s="2"/>
@@ -17626,13 +17657,13 @@
         <v>vitongojiphcc</v>
       </c>
       <c r="C55" s="2" t="s">
-        <v>1109</v>
+        <v>1111</v>
       </c>
       <c r="D55" s="2" t="s">
-        <v>1109</v>
+        <v>1111</v>
       </c>
       <c r="E55" s="2" t="s">
-        <v>1097</v>
+        <v>1099</v>
       </c>
       <c r="F55" s="2"/>
       <c r="G55" s="2"/>
@@ -17665,13 +17696,13 @@
         <v>weshaphcu+</v>
       </c>
       <c r="C56" s="2" t="s">
-        <v>1110</v>
+        <v>1112</v>
       </c>
       <c r="D56" s="2" t="s">
-        <v>1110</v>
+        <v>1112</v>
       </c>
       <c r="E56" s="2" t="s">
-        <v>1097</v>
+        <v>1099</v>
       </c>
       <c r="F56" s="2"/>
       <c r="G56" s="2"/>
@@ -17704,13 +17735,13 @@
         <v>kondephcu+</v>
       </c>
       <c r="C57" s="2" t="s">
-        <v>1111</v>
+        <v>1113</v>
       </c>
       <c r="D57" s="2" t="s">
-        <v>1111</v>
+        <v>1113</v>
       </c>
       <c r="E57" s="2" t="s">
-        <v>1099</v>
+        <v>1101</v>
       </c>
       <c r="F57" s="2"/>
       <c r="G57" s="2"/>
@@ -17743,13 +17774,13 @@
         <v>makangalephcu+</v>
       </c>
       <c r="C58" s="5" t="s">
-        <v>1112</v>
+        <v>1114</v>
       </c>
       <c r="D58" s="5" t="s">
-        <v>1112</v>
+        <v>1114</v>
       </c>
       <c r="E58" s="2" t="s">
-        <v>1099</v>
+        <v>1101</v>
       </c>
       <c r="F58" s="2"/>
       <c r="G58" s="2"/>
@@ -17782,13 +17813,13 @@
         <v>maziwangombephcu+</v>
       </c>
       <c r="C59" s="5" t="s">
-        <v>1113</v>
+        <v>1115</v>
       </c>
       <c r="D59" s="5" t="s">
-        <v>1113</v>
+        <v>1115</v>
       </c>
       <c r="E59" s="2" t="s">
-        <v>1099</v>
+        <v>1101</v>
       </c>
       <c r="F59" s="2"/>
       <c r="G59" s="2"/>
@@ -17821,13 +17852,13 @@
         <v>micheweniphcc</v>
       </c>
       <c r="C60" s="5" t="s">
-        <v>1114</v>
+        <v>1116</v>
       </c>
       <c r="D60" s="5" t="s">
-        <v>1114</v>
+        <v>1116</v>
       </c>
       <c r="E60" s="2" t="s">
-        <v>1099</v>
+        <v>1101</v>
       </c>
       <c r="F60" s="2"/>
       <c r="G60" s="2"/>
@@ -17860,13 +17891,13 @@
         <v>wingwiphcu+</v>
       </c>
       <c r="C61" s="2" t="s">
-        <v>1115</v>
+        <v>1117</v>
       </c>
       <c r="D61" s="2" t="s">
-        <v>1115</v>
+        <v>1117</v>
       </c>
       <c r="E61" s="2" t="s">
-        <v>1099</v>
+        <v>1101</v>
       </c>
       <c r="F61" s="2"/>
       <c r="G61" s="2"/>
@@ -17899,13 +17930,13 @@
         <v>kiuyumbuyuniphcu+</v>
       </c>
       <c r="C62" s="5" t="s">
-        <v>1116</v>
+        <v>1118</v>
       </c>
       <c r="D62" s="5" t="s">
-        <v>1116</v>
+        <v>1118</v>
       </c>
       <c r="E62" s="2" t="s">
-        <v>1099</v>
+        <v>1101</v>
       </c>
       <c r="F62" s="2"/>
       <c r="G62" s="2"/>
@@ -17938,13 +17969,13 @@
         <v>bogoaphcu+</v>
       </c>
       <c r="C63" s="2" t="s">
-        <v>1117</v>
+        <v>1119</v>
       </c>
       <c r="D63" s="2" t="s">
-        <v>1117</v>
+        <v>1119</v>
       </c>
       <c r="E63" s="2" t="s">
-        <v>1101</v>
+        <v>1103</v>
       </c>
       <c r="F63" s="2"/>
       <c r="G63" s="2"/>
@@ -17977,13 +18008,13 @@
         <v>kengejaphcu+</v>
       </c>
       <c r="C64" s="2" t="s">
-        <v>1118</v>
+        <v>1120</v>
       </c>
       <c r="D64" s="2" t="s">
-        <v>1118</v>
+        <v>1120</v>
       </c>
       <c r="E64" s="2" t="s">
-        <v>1101</v>
+        <v>1103</v>
       </c>
       <c r="F64" s="2"/>
       <c r="G64" s="2"/>
@@ -18016,13 +18047,13 @@
         <v>abdallahmzeedistricthospital</v>
       </c>
       <c r="C65" s="5" t="s">
-        <v>1119</v>
+        <v>1121</v>
       </c>
       <c r="D65" s="5" t="s">
-        <v>1120</v>
+        <v>1122</v>
       </c>
       <c r="E65" s="2" t="s">
-        <v>1101</v>
+        <v>1103</v>
       </c>
       <c r="F65" s="2"/>
       <c r="G65" s="2"/>
@@ -18055,13 +18086,13 @@
         <v>michenzaniphcu+</v>
       </c>
       <c r="C66" s="5" t="s">
-        <v>1121</v>
+        <v>1123</v>
       </c>
       <c r="D66" s="5" t="s">
-        <v>1121</v>
+        <v>1123</v>
       </c>
       <c r="E66" s="2" t="s">
-        <v>1101</v>
+        <v>1103</v>
       </c>
       <c r="F66" s="2"/>
       <c r="G66" s="2"/>
@@ -18094,13 +18125,13 @@
         <v>fundophcu+</v>
       </c>
       <c r="C67" s="2" t="s">
-        <v>1122</v>
+        <v>1124</v>
       </c>
       <c r="D67" s="2" t="s">
-        <v>1122</v>
+        <v>1124</v>
       </c>
       <c r="E67" s="2" t="s">
-        <v>1103</v>
+        <v>1105</v>
       </c>
       <c r="F67" s="2"/>
       <c r="G67" s="2"/>
@@ -18133,13 +18164,13 @@
         <v>kojaniphcu+</v>
       </c>
       <c r="C68" s="2" t="s">
-        <v>1123</v>
+        <v>1125</v>
       </c>
       <c r="D68" s="2" t="s">
-        <v>1123</v>
+        <v>1125</v>
       </c>
       <c r="E68" s="2" t="s">
-        <v>1103</v>
+        <v>1105</v>
       </c>
       <c r="F68" s="2"/>
       <c r="G68" s="2"/>
@@ -18172,13 +18203,13 @@
         <v>makongeniphcu+</v>
       </c>
       <c r="C69" s="5" t="s">
-        <v>1124</v>
+        <v>1126</v>
       </c>
       <c r="D69" s="5" t="s">
-        <v>1124</v>
+        <v>1126</v>
       </c>
       <c r="E69" s="2" t="s">
-        <v>1103</v>
+        <v>1105</v>
       </c>
       <c r="F69" s="2"/>
       <c r="G69" s="2"/>
@@ -18211,13 +18242,13 @@
         <v>wetedistricthospital</v>
       </c>
       <c r="C70" s="5" t="s">
-        <v>1125</v>
+        <v>1127</v>
       </c>
       <c r="D70" s="5" t="s">
-        <v>1126</v>
+        <v>1128</v>
       </c>
       <c r="E70" s="2" t="s">
-        <v>1103</v>
+        <v>1105</v>
       </c>
       <c r="F70" s="2"/>
       <c r="G70" s="2"/>
@@ -18250,13 +18281,13 @@
         <v>mzambarauniphcu+</v>
       </c>
       <c r="C71" s="5" t="s">
-        <v>1127</v>
+        <v>1129</v>
       </c>
       <c r="D71" s="5" t="s">
-        <v>1127</v>
+        <v>1129</v>
       </c>
       <c r="E71" s="2" t="s">
-        <v>1103</v>
+        <v>1105</v>
       </c>
       <c r="F71" s="2"/>
       <c r="G71" s="2"/>
@@ -18289,13 +18320,13 @@
         <v>junguniphcu+</v>
       </c>
       <c r="C72" s="2" t="s">
-        <v>1128</v>
+        <v>1130</v>
       </c>
       <c r="D72" s="2" t="s">
-        <v>1128</v>
+        <v>1130</v>
       </c>
       <c r="E72" s="2" t="s">
-        <v>1103</v>
+        <v>1105</v>
       </c>
       <c r="F72" s="2"/>
       <c r="G72" s="2"/>
@@ -18328,13 +18359,13 @@
         <v>ukunjwiphcu+</v>
       </c>
       <c r="C73" s="2" t="s">
-        <v>1129</v>
+        <v>1131</v>
       </c>
       <c r="D73" s="2" t="s">
-        <v>1129</v>
+        <v>1131</v>
       </c>
       <c r="E73" s="2" t="s">
-        <v>1103</v>
+        <v>1105</v>
       </c>
       <c r="F73" s="2"/>
       <c r="G73" s="2"/>
@@ -18367,13 +18398,13 @@
         <v>uondwephcu+</v>
       </c>
       <c r="C74" s="2" t="s">
-        <v>1130</v>
+        <v>1132</v>
       </c>
       <c r="D74" s="2" t="s">
-        <v>1130</v>
+        <v>1132</v>
       </c>
       <c r="E74" s="2" t="s">
-        <v>1103</v>
+        <v>1105</v>
       </c>
       <c r="F74" s="2"/>
       <c r="G74" s="2"/>
@@ -18406,13 +18437,13 @@
         <v>chwakaphcu+</v>
       </c>
       <c r="C75" s="2" t="s">
-        <v>1131</v>
+        <v>1133</v>
       </c>
       <c r="D75" s="2" t="s">
-        <v>1131</v>
+        <v>1133</v>
       </c>
       <c r="E75" s="2" t="s">
-        <v>1087</v>
+        <v>1089</v>
       </c>
       <c r="F75" s="2"/>
       <c r="G75" s="2"/>
@@ -18445,13 +18476,13 @@
         <v>mweraphcu+</v>
       </c>
       <c r="C76" s="2" t="s">
-        <v>1132</v>
+        <v>1134</v>
       </c>
       <c r="D76" s="2" t="s">
-        <v>1132</v>
+        <v>1134</v>
       </c>
       <c r="E76" s="2" t="s">
-        <v>1087</v>
+        <v>1089</v>
       </c>
       <c r="F76" s="2"/>
       <c r="G76" s="2"/>
@@ -18484,13 +18515,13 @@
         <v>ungujaukuuphcu+</v>
       </c>
       <c r="C77" s="5" t="s">
-        <v>1133</v>
+        <v>1135</v>
       </c>
       <c r="D77" s="5" t="s">
-        <v>1133</v>
+        <v>1135</v>
       </c>
       <c r="E77" s="2" t="s">
-        <v>1087</v>
+        <v>1089</v>
       </c>
       <c r="F77" s="2"/>
       <c r="G77" s="2"/>
@@ -18523,13 +18554,13 @@
         <v>uziniphcu+</v>
       </c>
       <c r="C78" s="2" t="s">
-        <v>1134</v>
+        <v>1136</v>
       </c>
       <c r="D78" s="2" t="s">
-        <v>1134</v>
+        <v>1136</v>
       </c>
       <c r="E78" s="2" t="s">
-        <v>1087</v>
+        <v>1089</v>
       </c>
       <c r="F78" s="2"/>
       <c r="G78" s="2"/>
@@ -18562,13 +18593,13 @@
         <v>uroaphcu+</v>
       </c>
       <c r="C79" s="2" t="s">
-        <v>1135</v>
+        <v>1137</v>
       </c>
       <c r="D79" s="2" t="s">
-        <v>1135</v>
+        <v>1137</v>
       </c>
       <c r="E79" s="2" t="s">
-        <v>1087</v>
+        <v>1089</v>
       </c>
       <c r="F79" s="2"/>
       <c r="G79" s="2"/>
@@ -18601,13 +18632,13 @@
         <v>kivungedistricthospital</v>
       </c>
       <c r="C80" s="5" t="s">
-        <v>1136</v>
+        <v>1138</v>
       </c>
       <c r="D80" s="2" t="s">
-        <v>1137</v>
+        <v>1139</v>
       </c>
       <c r="E80" s="2" t="s">
-        <v>1083</v>
+        <v>1085</v>
       </c>
       <c r="F80" s="2"/>
       <c r="G80" s="2"/>
@@ -18640,13 +18671,13 @@
         <v>matemwephcu+</v>
       </c>
       <c r="C81" s="5" t="s">
-        <v>1138</v>
+        <v>1140</v>
       </c>
       <c r="D81" s="5" t="s">
-        <v>1138</v>
+        <v>1140</v>
       </c>
       <c r="E81" s="2" t="s">
-        <v>1083</v>
+        <v>1085</v>
       </c>
       <c r="F81" s="2"/>
       <c r="G81" s="2"/>
@@ -18679,13 +18710,13 @@
         <v>nungwiphcu+</v>
       </c>
       <c r="C82" s="2" t="s">
-        <v>1139</v>
+        <v>1141</v>
       </c>
       <c r="D82" s="2" t="s">
-        <v>1139</v>
+        <v>1141</v>
       </c>
       <c r="E82" s="2" t="s">
-        <v>1083</v>
+        <v>1085</v>
       </c>
       <c r="F82" s="2"/>
       <c r="G82" s="2"/>
@@ -18718,13 +18749,13 @@
         <v>pwanimchanganiphcu+</v>
       </c>
       <c r="C83" s="5" t="s">
-        <v>1140</v>
+        <v>1142</v>
       </c>
       <c r="D83" s="5" t="s">
-        <v>1140</v>
+        <v>1142</v>
       </c>
       <c r="E83" s="2" t="s">
-        <v>1083</v>
+        <v>1085</v>
       </c>
       <c r="F83" s="2"/>
       <c r="G83" s="2"/>
@@ -18757,13 +18788,13 @@
         <v>tumbatugomaniphcu+</v>
       </c>
       <c r="C84" s="5" t="s">
-        <v>1141</v>
+        <v>1143</v>
       </c>
       <c r="D84" s="5" t="s">
-        <v>1141</v>
+        <v>1143</v>
       </c>
       <c r="E84" s="2" t="s">
-        <v>1083</v>
+        <v>1085</v>
       </c>
       <c r="F84" s="2"/>
       <c r="G84" s="2"/>
@@ -18796,13 +18827,13 @@
         <v>kendwaphcu+</v>
       </c>
       <c r="C85" s="2" t="s">
-        <v>1142</v>
+        <v>1144</v>
       </c>
       <c r="D85" s="2" t="s">
-        <v>1142</v>
+        <v>1144</v>
       </c>
       <c r="E85" s="2" t="s">
-        <v>1083</v>
+        <v>1085</v>
       </c>
       <c r="F85" s="2"/>
       <c r="G85" s="2"/>
@@ -18835,13 +18866,13 @@
         <v>bumbwinimisufiniphcu+</v>
       </c>
       <c r="C86" s="5" t="s">
-        <v>1143</v>
+        <v>1145</v>
       </c>
       <c r="D86" s="5" t="s">
-        <v>1143</v>
+        <v>1145</v>
       </c>
       <c r="E86" s="2" t="s">
-        <v>1085</v>
+        <v>1087</v>
       </c>
       <c r="F86" s="2"/>
       <c r="G86" s="2"/>
@@ -18874,13 +18905,13 @@
         <v>dongevijibweniphcu+</v>
       </c>
       <c r="C87" s="5" t="s">
-        <v>1144</v>
+        <v>1146</v>
       </c>
       <c r="D87" s="5" t="s">
-        <v>1144</v>
+        <v>1146</v>
       </c>
       <c r="E87" s="2" t="s">
-        <v>1085</v>
+        <v>1087</v>
       </c>
       <c r="F87" s="2"/>
       <c r="G87" s="2"/>
@@ -18913,13 +18944,13 @@
         <v>kiongwephcu</v>
       </c>
       <c r="C88" s="2" t="s">
-        <v>1145</v>
+        <v>1147</v>
       </c>
       <c r="D88" s="2" t="s">
-        <v>1145</v>
+        <v>1147</v>
       </c>
       <c r="E88" s="2" t="s">
-        <v>1085</v>
+        <v>1087</v>
       </c>
       <c r="F88" s="2"/>
       <c r="G88" s="2"/>
@@ -18952,13 +18983,13 @@
         <v>kitopephcu</v>
       </c>
       <c r="C89" s="2" t="s">
-        <v>1146</v>
+        <v>1148</v>
       </c>
       <c r="D89" s="2" t="s">
-        <v>1146</v>
+        <v>1148</v>
       </c>
       <c r="E89" s="2" t="s">
-        <v>1085</v>
+        <v>1087</v>
       </c>
       <c r="F89" s="2"/>
       <c r="G89" s="2"/>
@@ -18991,13 +19022,13 @@
         <v>mahondaphcu+</v>
       </c>
       <c r="C90" s="5" t="s">
-        <v>1147</v>
+        <v>1149</v>
       </c>
       <c r="D90" s="5" t="s">
-        <v>1147</v>
+        <v>1149</v>
       </c>
       <c r="E90" s="2" t="s">
-        <v>1085</v>
+        <v>1087</v>
       </c>
       <c r="F90" s="2"/>
       <c r="G90" s="2"/>
@@ -19030,13 +19061,13 @@
         <v>jambianiphcu+</v>
       </c>
       <c r="C91" s="5" t="s">
-        <v>1148</v>
+        <v>1150</v>
       </c>
       <c r="D91" s="5" t="s">
-        <v>1148</v>
+        <v>1150</v>
       </c>
       <c r="E91" s="2" t="s">
-        <v>1089</v>
+        <v>1091</v>
       </c>
       <c r="F91" s="2"/>
       <c r="G91" s="2"/>
@@ -19069,13 +19100,13 @@
         <v>makunduchidistricthospital</v>
       </c>
       <c r="C92" s="5" t="s">
-        <v>1149</v>
+        <v>1151</v>
       </c>
       <c r="D92" s="2" t="s">
-        <v>1150</v>
+        <v>1152</v>
       </c>
       <c r="E92" s="2" t="s">
-        <v>1089</v>
+        <v>1091</v>
       </c>
       <c r="F92" s="2"/>
       <c r="G92" s="2"/>
@@ -19108,13 +19139,13 @@
         <v>muyuniphcu+</v>
       </c>
       <c r="C93" s="2" t="s">
-        <v>1151</v>
+        <v>1153</v>
       </c>
       <c r="D93" s="2" t="s">
-        <v>1151</v>
+        <v>1153</v>
       </c>
       <c r="E93" s="2" t="s">
-        <v>1089</v>
+        <v>1091</v>
       </c>
       <c r="F93" s="2"/>
       <c r="G93" s="2"/>
@@ -19147,13 +19178,13 @@
         <v>bwejuuphcu+</v>
       </c>
       <c r="C94" s="2" t="s">
-        <v>1152</v>
+        <v>1154</v>
       </c>
       <c r="D94" s="2" t="s">
-        <v>1152</v>
+        <v>1154</v>
       </c>
       <c r="E94" s="2" t="s">
-        <v>1089</v>
+        <v>1091</v>
       </c>
       <c r="F94" s="2"/>
       <c r="G94" s="2"/>
@@ -19186,13 +19217,13 @@
         <v>chumbuniphcu+</v>
       </c>
       <c r="C95" s="5" t="s">
-        <v>1153</v>
+        <v>1155</v>
       </c>
       <c r="D95" s="5" t="s">
-        <v>1153</v>
+        <v>1155</v>
       </c>
       <c r="E95" s="2" t="s">
-        <v>1095</v>
+        <v>1097</v>
       </c>
       <c r="F95" s="2"/>
       <c r="G95" s="2"/>
@@ -19225,13 +19256,13 @@
         <v>mnazimmojahospital</v>
       </c>
       <c r="C96" s="5" t="s">
-        <v>1154</v>
+        <v>1156</v>
       </c>
       <c r="D96" s="2" t="s">
-        <v>1155</v>
+        <v>1157</v>
       </c>
       <c r="E96" s="2" t="s">
-        <v>1095</v>
+        <v>1097</v>
       </c>
       <c r="F96" s="2"/>
       <c r="G96" s="2"/>
@@ -19264,13 +19295,13 @@
         <v>mwembeladumchclinic</v>
       </c>
       <c r="C97" s="5" t="s">
-        <v>1156</v>
+        <v>1158</v>
       </c>
       <c r="D97" s="2" t="s">
-        <v>1157</v>
+        <v>1159</v>
       </c>
       <c r="E97" s="2" t="s">
-        <v>1095</v>
+        <v>1097</v>
       </c>
       <c r="F97" s="2"/>
       <c r="G97" s="2"/>
@@ -19303,13 +19334,13 @@
         <v>sebleniphcu+</v>
       </c>
       <c r="C98" s="2" t="s">
-        <v>1158</v>
+        <v>1160</v>
       </c>
       <c r="D98" s="2" t="s">
-        <v>1158</v>
+        <v>1160</v>
       </c>
       <c r="E98" s="2" t="s">
-        <v>1095</v>
+        <v>1097</v>
       </c>
       <c r="F98" s="2"/>
       <c r="G98" s="2"/>
@@ -19342,13 +19373,13 @@
         <v>chukwaniphcu+</v>
       </c>
       <c r="C99" s="5" t="s">
-        <v>1159</v>
+        <v>1161</v>
       </c>
       <c r="D99" s="5" t="s">
-        <v>1159</v>
+        <v>1161</v>
       </c>
       <c r="E99" s="2" t="s">
-        <v>1093</v>
+        <v>1095</v>
       </c>
       <c r="F99" s="2"/>
       <c r="G99" s="2"/>
@@ -19381,13 +19412,13 @@
         <v>fuoniphcu+</v>
       </c>
       <c r="C100" s="2" t="s">
-        <v>1160</v>
+        <v>1162</v>
       </c>
       <c r="D100" s="2" t="s">
-        <v>1160</v>
+        <v>1162</v>
       </c>
       <c r="E100" s="2" t="s">
-        <v>1093</v>
+        <v>1095</v>
       </c>
       <c r="F100" s="2"/>
       <c r="G100" s="2"/>
@@ -19420,13 +19451,13 @@
         <v>kombeniphcu+</v>
       </c>
       <c r="C101" s="5" t="s">
-        <v>1161</v>
+        <v>1163</v>
       </c>
       <c r="D101" s="5" t="s">
-        <v>1161</v>
+        <v>1163</v>
       </c>
       <c r="E101" s="2" t="s">
-        <v>1093</v>
+        <v>1095</v>
       </c>
       <c r="F101" s="2"/>
       <c r="G101" s="2"/>
@@ -19459,13 +19490,13 @@
         <v>mtofaaniphcu+(kinuni)</v>
       </c>
       <c r="C102" s="5" t="s">
-        <v>1162</v>
+        <v>1164</v>
       </c>
       <c r="D102" s="5" t="s">
-        <v>1162</v>
+        <v>1164</v>
       </c>
       <c r="E102" s="2" t="s">
-        <v>1091</v>
+        <v>1093</v>
       </c>
       <c r="F102" s="2"/>
       <c r="G102" s="2"/>
@@ -19498,13 +19529,13 @@
         <v>bumbwisudiphcu+</v>
       </c>
       <c r="C103" s="5" t="s">
-        <v>1163</v>
+        <v>1165</v>
       </c>
       <c r="D103" s="5" t="s">
-        <v>1163</v>
+        <v>1165</v>
       </c>
       <c r="E103" s="2" t="s">
-        <v>1091</v>
+        <v>1093</v>
       </c>
       <c r="F103" s="2"/>
       <c r="G103" s="2"/>
@@ -19537,13 +19568,13 @@
         <v>selemphcu+</v>
       </c>
       <c r="C104" s="2" t="s">
-        <v>1164</v>
+        <v>1166</v>
       </c>
       <c r="D104" s="2" t="s">
-        <v>1164</v>
+        <v>1166</v>
       </c>
       <c r="E104" s="2" t="s">
-        <v>1091</v>
+        <v>1093</v>
       </c>
       <c r="F104" s="2"/>
       <c r="G104" s="2"/>
@@ -19576,13 +19607,13 @@
         <v>other</v>
       </c>
       <c r="C105" s="2" t="s">
-        <v>1081</v>
+        <v>1083</v>
       </c>
       <c r="D105" s="2" t="s">
-        <v>1165</v>
+        <v>1167</v>
       </c>
       <c r="E105" s="2" t="s">
-        <v>1097</v>
+        <v>1099</v>
       </c>
       <c r="F105" s="2"/>
       <c r="G105" s="2"/>
@@ -19615,13 +19646,13 @@
         <v>other</v>
       </c>
       <c r="C106" s="2" t="s">
-        <v>1081</v>
+        <v>1083</v>
       </c>
       <c r="D106" s="2" t="s">
-        <v>1165</v>
+        <v>1167</v>
       </c>
       <c r="E106" s="2" t="s">
-        <v>1099</v>
+        <v>1101</v>
       </c>
       <c r="F106" s="2"/>
       <c r="G106" s="2"/>
@@ -19654,13 +19685,13 @@
         <v>other</v>
       </c>
       <c r="C107" s="2" t="s">
-        <v>1081</v>
+        <v>1083</v>
       </c>
       <c r="D107" s="2" t="s">
-        <v>1165</v>
+        <v>1167</v>
       </c>
       <c r="E107" s="2" t="s">
-        <v>1101</v>
+        <v>1103</v>
       </c>
       <c r="F107" s="2"/>
       <c r="G107" s="2"/>
@@ -19693,13 +19724,13 @@
         <v>other</v>
       </c>
       <c r="C108" s="2" t="s">
-        <v>1081</v>
+        <v>1083</v>
       </c>
       <c r="D108" s="2" t="s">
-        <v>1165</v>
+        <v>1167</v>
       </c>
       <c r="E108" s="2" t="s">
-        <v>1103</v>
+        <v>1105</v>
       </c>
       <c r="F108" s="2"/>
       <c r="G108" s="2"/>
@@ -19732,13 +19763,13 @@
         <v>other</v>
       </c>
       <c r="C109" s="2" t="s">
-        <v>1081</v>
+        <v>1083</v>
       </c>
       <c r="D109" s="2" t="s">
-        <v>1165</v>
+        <v>1167</v>
       </c>
       <c r="E109" s="2" t="s">
-        <v>1087</v>
+        <v>1089</v>
       </c>
       <c r="F109" s="2"/>
       <c r="G109" s="2"/>
@@ -19771,13 +19802,13 @@
         <v>other</v>
       </c>
       <c r="C110" s="2" t="s">
-        <v>1081</v>
+        <v>1083</v>
       </c>
       <c r="D110" s="2" t="s">
-        <v>1165</v>
+        <v>1167</v>
       </c>
       <c r="E110" s="2" t="s">
-        <v>1083</v>
+        <v>1085</v>
       </c>
       <c r="F110" s="2"/>
       <c r="G110" s="2"/>
@@ -19810,13 +19841,13 @@
         <v>other</v>
       </c>
       <c r="C111" s="2" t="s">
-        <v>1081</v>
+        <v>1083</v>
       </c>
       <c r="D111" s="2" t="s">
-        <v>1165</v>
+        <v>1167</v>
       </c>
       <c r="E111" s="2" t="s">
-        <v>1085</v>
+        <v>1087</v>
       </c>
       <c r="F111" s="2"/>
       <c r="G111" s="2"/>
@@ -19849,13 +19880,13 @@
         <v>other</v>
       </c>
       <c r="C112" s="2" t="s">
-        <v>1081</v>
+        <v>1083</v>
       </c>
       <c r="D112" s="2" t="s">
-        <v>1165</v>
+        <v>1167</v>
       </c>
       <c r="E112" s="2" t="s">
-        <v>1089</v>
+        <v>1091</v>
       </c>
       <c r="F112" s="2"/>
       <c r="G112" s="2"/>
@@ -19888,13 +19919,13 @@
         <v>other</v>
       </c>
       <c r="C113" s="2" t="s">
-        <v>1081</v>
+        <v>1083</v>
       </c>
       <c r="D113" s="2" t="s">
-        <v>1165</v>
+        <v>1167</v>
       </c>
       <c r="E113" s="2" t="s">
-        <v>1095</v>
+        <v>1097</v>
       </c>
       <c r="F113" s="2"/>
       <c r="G113" s="2"/>
@@ -19927,13 +19958,13 @@
         <v>other</v>
       </c>
       <c r="C114" s="2" t="s">
-        <v>1081</v>
+        <v>1083</v>
       </c>
       <c r="D114" s="2" t="s">
-        <v>1165</v>
+        <v>1167</v>
       </c>
       <c r="E114" s="2" t="s">
-        <v>1093</v>
+        <v>1095</v>
       </c>
       <c r="F114" s="2"/>
       <c r="G114" s="2"/>
@@ -19966,13 +19997,13 @@
         <v>other</v>
       </c>
       <c r="C115" s="2" t="s">
-        <v>1081</v>
+        <v>1083</v>
       </c>
       <c r="D115" s="2" t="s">
-        <v>1165</v>
+        <v>1167</v>
       </c>
       <c r="E115" s="2" t="s">
-        <v>1091</v>
+        <v>1093</v>
       </c>
       <c r="F115" s="2"/>
       <c r="G115" s="2"/>
@@ -20004,10 +20035,10 @@
         <v>139</v>
       </c>
       <c r="C116" s="4" t="s">
-        <v>1166</v>
+        <v>1168</v>
       </c>
       <c r="D116" s="2" t="s">
-        <v>1167</v>
+        <v>1169</v>
       </c>
     </row>
     <row r="117" customFormat="false" ht="13" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20015,13 +20046,13 @@
         <v>744</v>
       </c>
       <c r="B117" s="4" t="s">
-        <v>1168</v>
+        <v>1170</v>
       </c>
       <c r="C117" s="14" t="s">
-        <v>1169</v>
+        <v>1171</v>
       </c>
       <c r="D117" s="5" t="s">
-        <v>1170</v>
+        <v>1172</v>
       </c>
     </row>
     <row r="118" customFormat="false" ht="13" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20029,97 +20060,97 @@
         <v>744</v>
       </c>
       <c r="B118" s="4" t="s">
-        <v>971</v>
+        <v>973</v>
       </c>
       <c r="C118" s="4" t="s">
-        <v>1171</v>
+        <v>1173</v>
       </c>
       <c r="D118" s="2" t="s">
-        <v>1172</v>
+        <v>1174</v>
       </c>
     </row>
     <row r="119" customFormat="false" ht="13" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A119" s="4" t="s">
-        <v>1173</v>
+        <v>1175</v>
       </c>
       <c r="B119" s="4" t="s">
-        <v>1174</v>
+        <v>1176</v>
       </c>
       <c r="C119" s="4" t="s">
-        <v>1175</v>
+        <v>1177</v>
       </c>
       <c r="D119" s="2" t="s">
-        <v>1176</v>
+        <v>1178</v>
       </c>
     </row>
     <row r="120" customFormat="false" ht="13" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A120" s="4" t="s">
-        <v>1173</v>
+        <v>1175</v>
       </c>
       <c r="B120" s="4" t="s">
-        <v>1177</v>
+        <v>1179</v>
       </c>
       <c r="C120" s="4" t="s">
-        <v>1178</v>
+        <v>1180</v>
       </c>
       <c r="D120" s="2" t="s">
-        <v>1179</v>
+        <v>1181</v>
       </c>
     </row>
     <row r="121" customFormat="false" ht="13" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A121" s="4" t="s">
-        <v>1173</v>
+        <v>1175</v>
       </c>
       <c r="B121" s="4" t="s">
-        <v>1180</v>
+        <v>1182</v>
       </c>
       <c r="C121" s="14" t="s">
-        <v>1181</v>
+        <v>1183</v>
       </c>
       <c r="D121" s="2" t="s">
-        <v>1182</v>
+        <v>1184</v>
       </c>
     </row>
     <row r="122" customFormat="false" ht="13" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A122" s="4" t="s">
-        <v>1173</v>
+        <v>1175</v>
       </c>
       <c r="B122" s="4" t="s">
-        <v>1183</v>
+        <v>1185</v>
       </c>
       <c r="C122" s="14" t="s">
-        <v>1184</v>
+        <v>1186</v>
       </c>
       <c r="D122" s="5" t="s">
-        <v>1185</v>
+        <v>1187</v>
       </c>
     </row>
     <row r="123" customFormat="false" ht="13" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A123" s="4" t="s">
-        <v>1173</v>
+        <v>1175</v>
       </c>
       <c r="B123" s="4" t="s">
-        <v>1186</v>
+        <v>1188</v>
       </c>
       <c r="C123" s="4" t="s">
-        <v>1187</v>
+        <v>1189</v>
       </c>
       <c r="D123" s="2" t="s">
-        <v>1188</v>
+        <v>1190</v>
       </c>
     </row>
     <row r="124" customFormat="false" ht="13" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A124" s="4" t="s">
-        <v>1173</v>
+        <v>1175</v>
       </c>
       <c r="B124" s="4" t="s">
-        <v>1080</v>
+        <v>1082</v>
       </c>
       <c r="C124" s="4" t="s">
-        <v>1081</v>
+        <v>1083</v>
       </c>
       <c r="D124" s="2" t="s">
-        <v>1189</v>
+        <v>1191</v>
       </c>
     </row>
     <row r="125" customFormat="false" ht="13" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20127,13 +20158,13 @@
         <v>753</v>
       </c>
       <c r="B125" s="4" t="s">
-        <v>1190</v>
+        <v>1192</v>
       </c>
       <c r="C125" s="4" t="s">
-        <v>1191</v>
+        <v>1193</v>
       </c>
       <c r="D125" s="2" t="s">
-        <v>1192</v>
+        <v>1194</v>
       </c>
     </row>
     <row r="126" customFormat="false" ht="13" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20141,13 +20172,13 @@
         <v>753</v>
       </c>
       <c r="B126" s="4" t="s">
-        <v>1193</v>
+        <v>1195</v>
       </c>
       <c r="C126" s="4" t="s">
-        <v>1194</v>
+        <v>1196</v>
       </c>
       <c r="D126" s="2" t="s">
-        <v>1195</v>
+        <v>1197</v>
       </c>
     </row>
     <row r="127" customFormat="false" ht="13" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20155,13 +20186,13 @@
         <v>753</v>
       </c>
       <c r="B127" s="4" t="s">
-        <v>1196</v>
+        <v>1198</v>
       </c>
       <c r="C127" s="4" t="s">
-        <v>1197</v>
+        <v>1199</v>
       </c>
       <c r="D127" s="2" t="s">
-        <v>1198</v>
+        <v>1200</v>
       </c>
     </row>
     <row r="128" customFormat="false" ht="13" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20169,13 +20200,13 @@
         <v>753</v>
       </c>
       <c r="B128" s="4" t="s">
-        <v>1199</v>
+        <v>1201</v>
       </c>
       <c r="C128" s="4" t="s">
-        <v>1200</v>
+        <v>1202</v>
       </c>
       <c r="D128" s="2" t="s">
-        <v>1201</v>
+        <v>1203</v>
       </c>
     </row>
     <row r="129" customFormat="false" ht="13" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20183,13 +20214,13 @@
         <v>753</v>
       </c>
       <c r="B129" s="4" t="s">
-        <v>1202</v>
+        <v>1204</v>
       </c>
       <c r="C129" s="4" t="s">
-        <v>1203</v>
+        <v>1205</v>
       </c>
       <c r="D129" s="2" t="s">
-        <v>1204</v>
+        <v>1206</v>
       </c>
     </row>
     <row r="130" customFormat="false" ht="13" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20197,13 +20228,13 @@
         <v>753</v>
       </c>
       <c r="B130" s="4" t="s">
-        <v>1205</v>
+        <v>1207</v>
       </c>
       <c r="C130" s="4" t="s">
-        <v>1206</v>
+        <v>1208</v>
       </c>
       <c r="D130" s="2" t="s">
-        <v>1206</v>
+        <v>1208</v>
       </c>
     </row>
     <row r="131" customFormat="false" ht="13" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20211,13 +20242,13 @@
         <v>753</v>
       </c>
       <c r="B131" s="4" t="s">
-        <v>1080</v>
+        <v>1082</v>
       </c>
       <c r="C131" s="4" t="s">
-        <v>1081</v>
+        <v>1083</v>
       </c>
       <c r="D131" s="2" t="s">
-        <v>1189</v>
+        <v>1191</v>
       </c>
     </row>
     <row r="132" customFormat="false" ht="13" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20225,13 +20256,13 @@
         <v>758</v>
       </c>
       <c r="B132" s="4" t="s">
-        <v>1207</v>
+        <v>1209</v>
       </c>
       <c r="C132" s="4" t="s">
-        <v>1208</v>
+        <v>1210</v>
       </c>
       <c r="D132" s="2" t="s">
-        <v>1209</v>
+        <v>1211</v>
       </c>
     </row>
     <row r="133" customFormat="false" ht="13" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20239,13 +20270,13 @@
         <v>758</v>
       </c>
       <c r="B133" s="4" t="s">
-        <v>1210</v>
+        <v>1212</v>
       </c>
       <c r="C133" s="4" t="s">
-        <v>1211</v>
+        <v>1213</v>
       </c>
       <c r="D133" s="2" t="s">
-        <v>1212</v>
+        <v>1214</v>
       </c>
     </row>
     <row r="134" customFormat="false" ht="13" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20253,13 +20284,13 @@
         <v>758</v>
       </c>
       <c r="B134" s="4" t="s">
-        <v>1213</v>
+        <v>1215</v>
       </c>
       <c r="C134" s="4" t="s">
-        <v>1214</v>
+        <v>1216</v>
       </c>
       <c r="D134" s="2" t="s">
-        <v>1215</v>
+        <v>1217</v>
       </c>
     </row>
     <row r="135" customFormat="false" ht="13" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20270,10 +20301,10 @@
         <v>526</v>
       </c>
       <c r="C135" s="4" t="s">
-        <v>1216</v>
+        <v>1218</v>
       </c>
       <c r="D135" s="2" t="s">
-        <v>1217</v>
+        <v>1219</v>
       </c>
     </row>
     <row r="136" customFormat="false" ht="13" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20281,13 +20312,13 @@
         <v>758</v>
       </c>
       <c r="B136" s="4" t="s">
-        <v>1218</v>
+        <v>1220</v>
       </c>
       <c r="C136" s="4" t="s">
-        <v>1219</v>
+        <v>1221</v>
       </c>
       <c r="D136" s="2" t="s">
-        <v>1220</v>
+        <v>1222</v>
       </c>
     </row>
     <row r="137" customFormat="false" ht="13" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20295,13 +20326,13 @@
         <v>758</v>
       </c>
       <c r="B137" s="4" t="s">
-        <v>1202</v>
+        <v>1204</v>
       </c>
       <c r="C137" s="4" t="s">
-        <v>1221</v>
+        <v>1223</v>
       </c>
       <c r="D137" s="2" t="s">
-        <v>1204</v>
+        <v>1206</v>
       </c>
     </row>
     <row r="138" customFormat="false" ht="13" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20309,13 +20340,13 @@
         <v>758</v>
       </c>
       <c r="B138" s="4" t="s">
-        <v>1222</v>
+        <v>1224</v>
       </c>
       <c r="C138" s="4" t="s">
-        <v>1223</v>
+        <v>1225</v>
       </c>
       <c r="D138" s="2" t="s">
-        <v>1198</v>
+        <v>1200</v>
       </c>
     </row>
     <row r="139" customFormat="false" ht="13" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20323,13 +20354,13 @@
         <v>758</v>
       </c>
       <c r="B139" s="4" t="s">
-        <v>1224</v>
+        <v>1226</v>
       </c>
       <c r="C139" s="4" t="s">
-        <v>1225</v>
+        <v>1227</v>
       </c>
       <c r="D139" s="2" t="s">
-        <v>1226</v>
+        <v>1228</v>
       </c>
     </row>
     <row r="140" customFormat="false" ht="13" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20337,13 +20368,13 @@
         <v>758</v>
       </c>
       <c r="B140" s="4" t="s">
-        <v>1227</v>
+        <v>1229</v>
       </c>
       <c r="C140" s="4" t="s">
-        <v>1228</v>
+        <v>1230</v>
       </c>
       <c r="D140" s="2" t="s">
-        <v>1229</v>
+        <v>1231</v>
       </c>
     </row>
     <row r="141" customFormat="false" ht="13" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20351,13 +20382,13 @@
         <v>758</v>
       </c>
       <c r="B141" s="4" t="s">
-        <v>1230</v>
+        <v>1232</v>
       </c>
       <c r="C141" s="4" t="s">
-        <v>1231</v>
+        <v>1233</v>
       </c>
       <c r="D141" s="2" t="s">
-        <v>1232</v>
+        <v>1234</v>
       </c>
     </row>
     <row r="142" customFormat="false" ht="13" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20365,13 +20396,13 @@
         <v>773</v>
       </c>
       <c r="B142" s="4" t="s">
-        <v>1233</v>
+        <v>1235</v>
       </c>
       <c r="C142" s="4" t="s">
-        <v>1234</v>
+        <v>1236</v>
       </c>
       <c r="D142" s="2" t="s">
-        <v>1235</v>
+        <v>1237</v>
       </c>
     </row>
     <row r="143" customFormat="false" ht="13" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20379,13 +20410,13 @@
         <v>773</v>
       </c>
       <c r="B143" s="4" t="s">
-        <v>1196</v>
+        <v>1198</v>
       </c>
       <c r="C143" s="4" t="s">
-        <v>1236</v>
+        <v>1238</v>
       </c>
       <c r="D143" s="2" t="s">
-        <v>1198</v>
+        <v>1200</v>
       </c>
     </row>
     <row r="144" customFormat="false" ht="13" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20393,13 +20424,13 @@
         <v>773</v>
       </c>
       <c r="B144" s="4" t="s">
-        <v>1237</v>
+        <v>1239</v>
       </c>
       <c r="C144" s="4" t="s">
-        <v>1238</v>
+        <v>1240</v>
       </c>
       <c r="D144" s="2" t="s">
-        <v>1239</v>
+        <v>1241</v>
       </c>
     </row>
     <row r="145" customFormat="false" ht="13" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20410,10 +20441,10 @@
         <v>342</v>
       </c>
       <c r="C145" s="4" t="s">
-        <v>1240</v>
+        <v>1242</v>
       </c>
       <c r="D145" s="2" t="s">
-        <v>1241</v>
+        <v>1243</v>
       </c>
     </row>
     <row r="146" customFormat="false" ht="13" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20421,13 +20452,13 @@
         <v>773</v>
       </c>
       <c r="B146" s="4" t="s">
-        <v>1242</v>
+        <v>1244</v>
       </c>
       <c r="C146" s="4" t="s">
-        <v>1243</v>
+        <v>1245</v>
       </c>
       <c r="D146" s="2" t="s">
-        <v>1244</v>
+        <v>1246</v>
       </c>
     </row>
     <row r="147" customFormat="false" ht="13" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20435,13 +20466,13 @@
         <v>773</v>
       </c>
       <c r="B147" s="4" t="s">
-        <v>1080</v>
+        <v>1082</v>
       </c>
       <c r="C147" s="4" t="s">
-        <v>1080</v>
+        <v>1082</v>
       </c>
       <c r="D147" s="2" t="s">
-        <v>1245</v>
+        <v>1247</v>
       </c>
     </row>
     <row r="148" customFormat="false" ht="13" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20449,13 +20480,13 @@
         <v>777</v>
       </c>
       <c r="B148" s="4" t="s">
-        <v>1246</v>
+        <v>1248</v>
       </c>
       <c r="C148" s="4" t="s">
-        <v>1246</v>
+        <v>1248</v>
       </c>
       <c r="D148" s="2" t="s">
-        <v>1247</v>
+        <v>1249</v>
       </c>
     </row>
     <row r="149" customFormat="false" ht="13" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20463,13 +20494,13 @@
         <v>777</v>
       </c>
       <c r="B149" s="4" t="s">
-        <v>1248</v>
+        <v>1250</v>
       </c>
       <c r="C149" s="4" t="s">
-        <v>1249</v>
+        <v>1251</v>
       </c>
       <c r="D149" s="2" t="s">
-        <v>1250</v>
+        <v>1252</v>
       </c>
     </row>
     <row r="150" customFormat="false" ht="13" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20477,13 +20508,13 @@
         <v>777</v>
       </c>
       <c r="B150" s="4" t="s">
-        <v>1251</v>
+        <v>1253</v>
       </c>
       <c r="C150" s="4" t="s">
-        <v>1252</v>
+        <v>1254</v>
       </c>
       <c r="D150" s="2" t="s">
-        <v>1253</v>
+        <v>1255</v>
       </c>
     </row>
     <row r="151" customFormat="false" ht="13" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20491,13 +20522,13 @@
         <v>791</v>
       </c>
       <c r="B151" s="2" t="s">
-        <v>1254</v>
+        <v>1256</v>
       </c>
       <c r="C151" s="2" t="s">
-        <v>1255</v>
+        <v>1257</v>
       </c>
       <c r="D151" s="2" t="s">
-        <v>1256</v>
+        <v>1258</v>
       </c>
     </row>
     <row r="152" customFormat="false" ht="13" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20505,13 +20536,13 @@
         <v>791</v>
       </c>
       <c r="B152" s="2" t="s">
-        <v>1257</v>
+        <v>1259</v>
       </c>
       <c r="C152" s="2" t="s">
-        <v>1258</v>
+        <v>1260</v>
       </c>
       <c r="D152" s="2" t="s">
-        <v>1259</v>
+        <v>1261</v>
       </c>
     </row>
     <row r="153" customFormat="false" ht="13" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20519,13 +20550,13 @@
         <v>791</v>
       </c>
       <c r="B153" s="2" t="s">
-        <v>1260</v>
+        <v>1262</v>
       </c>
       <c r="C153" s="2" t="s">
-        <v>1261</v>
+        <v>1263</v>
       </c>
       <c r="D153" s="2" t="s">
-        <v>1262</v>
+        <v>1264</v>
       </c>
     </row>
     <row r="154" customFormat="false" ht="13" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20533,13 +20564,13 @@
         <v>791</v>
       </c>
       <c r="B154" s="2" t="s">
-        <v>1263</v>
+        <v>1265</v>
       </c>
       <c r="C154" s="2" t="s">
-        <v>1264</v>
+        <v>1266</v>
       </c>
       <c r="D154" s="2" t="s">
-        <v>1265</v>
+        <v>1267</v>
       </c>
     </row>
     <row r="155" customFormat="false" ht="13" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20547,13 +20578,13 @@
         <v>797</v>
       </c>
       <c r="B155" s="2" t="s">
-        <v>1266</v>
+        <v>1268</v>
       </c>
       <c r="C155" s="2" t="s">
-        <v>1267</v>
+        <v>1269</v>
       </c>
       <c r="D155" s="2" t="s">
-        <v>1268</v>
+        <v>1270</v>
       </c>
     </row>
     <row r="156" customFormat="false" ht="13" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20561,13 +20592,13 @@
         <v>797</v>
       </c>
       <c r="B156" s="2" t="s">
-        <v>1269</v>
+        <v>1271</v>
       </c>
       <c r="C156" s="2" t="s">
-        <v>1270</v>
+        <v>1272</v>
       </c>
       <c r="D156" s="2" t="s">
-        <v>1271</v>
+        <v>1273</v>
       </c>
     </row>
     <row r="157" customFormat="false" ht="13" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20575,13 +20606,13 @@
         <v>797</v>
       </c>
       <c r="B157" s="2" t="s">
-        <v>1272</v>
+        <v>1274</v>
       </c>
       <c r="C157" s="2" t="s">
-        <v>1273</v>
+        <v>1275</v>
       </c>
       <c r="D157" s="2" t="s">
-        <v>1274</v>
+        <v>1276</v>
       </c>
     </row>
     <row r="158" customFormat="false" ht="13" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20589,13 +20620,13 @@
         <v>797</v>
       </c>
       <c r="B158" s="2" t="s">
-        <v>1275</v>
+        <v>1277</v>
       </c>
       <c r="C158" s="2" t="s">
-        <v>1276</v>
+        <v>1278</v>
       </c>
       <c r="D158" s="2" t="s">
-        <v>1277</v>
+        <v>1279</v>
       </c>
     </row>
     <row r="159" customFormat="false" ht="13" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20603,13 +20634,13 @@
         <v>797</v>
       </c>
       <c r="B159" s="2" t="s">
-        <v>1278</v>
+        <v>1280</v>
       </c>
       <c r="C159" s="2" t="s">
-        <v>1279</v>
+        <v>1281</v>
       </c>
       <c r="D159" s="2" t="s">
-        <v>1280</v>
+        <v>1282</v>
       </c>
     </row>
     <row r="160" customFormat="false" ht="13" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20617,13 +20648,13 @@
         <v>797</v>
       </c>
       <c r="B160" s="2" t="s">
-        <v>1281</v>
+        <v>1283</v>
       </c>
       <c r="C160" s="2" t="s">
-        <v>1282</v>
+        <v>1284</v>
       </c>
       <c r="D160" s="2" t="s">
-        <v>1283</v>
+        <v>1285</v>
       </c>
     </row>
     <row r="161" customFormat="false" ht="13" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20631,13 +20662,13 @@
         <v>797</v>
       </c>
       <c r="B161" s="2" t="s">
-        <v>1284</v>
+        <v>1286</v>
       </c>
       <c r="C161" s="2" t="s">
-        <v>1285</v>
+        <v>1287</v>
       </c>
       <c r="D161" s="2" t="s">
-        <v>1286</v>
+        <v>1288</v>
       </c>
     </row>
     <row r="162" customFormat="false" ht="13" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20645,13 +20676,13 @@
         <v>797</v>
       </c>
       <c r="B162" s="2" t="s">
-        <v>1080</v>
+        <v>1082</v>
       </c>
       <c r="C162" s="2" t="s">
-        <v>1287</v>
+        <v>1289</v>
       </c>
       <c r="D162" s="2" t="s">
-        <v>1165</v>
+        <v>1167</v>
       </c>
     </row>
     <row r="163" customFormat="false" ht="13" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20659,13 +20690,13 @@
         <v>797</v>
       </c>
       <c r="B163" s="2" t="s">
-        <v>1288</v>
+        <v>1290</v>
       </c>
       <c r="C163" s="6" t="s">
-        <v>1289</v>
+        <v>1291</v>
       </c>
       <c r="D163" s="2" t="s">
-        <v>1265</v>
+        <v>1267</v>
       </c>
     </row>
     <row r="164" customFormat="false" ht="13" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20673,13 +20704,13 @@
         <v>173</v>
       </c>
       <c r="B164" s="2" t="s">
-        <v>1290</v>
+        <v>1292</v>
       </c>
       <c r="C164" s="29" t="s">
-        <v>1291</v>
+        <v>1293</v>
       </c>
       <c r="D164" s="2" t="s">
-        <v>1292</v>
+        <v>1294</v>
       </c>
     </row>
     <row r="165" customFormat="false" ht="13" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20687,13 +20718,13 @@
         <v>173</v>
       </c>
       <c r="B165" s="2" t="s">
-        <v>1293</v>
+        <v>1295</v>
       </c>
       <c r="C165" s="29" t="s">
-        <v>1294</v>
+        <v>1296</v>
       </c>
       <c r="D165" s="2" t="s">
-        <v>1295</v>
+        <v>1297</v>
       </c>
       <c r="E165" s="30"/>
     </row>
@@ -20702,13 +20733,13 @@
         <v>173</v>
       </c>
       <c r="B166" s="2" t="s">
-        <v>1296</v>
+        <v>1298</v>
       </c>
       <c r="C166" s="29" t="s">
-        <v>1297</v>
+        <v>1299</v>
       </c>
       <c r="D166" s="2" t="s">
-        <v>1298</v>
+        <v>1300</v>
       </c>
       <c r="E166" s="30"/>
     </row>
@@ -20717,13 +20748,13 @@
         <v>173</v>
       </c>
       <c r="B167" s="2" t="s">
-        <v>1299</v>
+        <v>1301</v>
       </c>
       <c r="C167" s="29" t="s">
-        <v>1300</v>
+        <v>1302</v>
       </c>
       <c r="D167" s="2" t="s">
-        <v>1301</v>
+        <v>1303</v>
       </c>
       <c r="E167" s="30"/>
     </row>
@@ -20732,13 +20763,13 @@
         <v>173</v>
       </c>
       <c r="B168" s="2" t="s">
-        <v>1302</v>
+        <v>1304</v>
       </c>
       <c r="C168" s="29" t="s">
-        <v>1303</v>
+        <v>1305</v>
       </c>
       <c r="D168" s="2" t="s">
-        <v>1304</v>
+        <v>1306</v>
       </c>
       <c r="E168" s="30"/>
     </row>
@@ -20747,13 +20778,13 @@
         <v>173</v>
       </c>
       <c r="B169" s="2" t="s">
-        <v>1305</v>
+        <v>1307</v>
       </c>
       <c r="C169" s="29" t="s">
-        <v>1306</v>
+        <v>1308</v>
       </c>
       <c r="D169" s="2" t="s">
-        <v>1307</v>
+        <v>1309</v>
       </c>
       <c r="E169" s="30"/>
     </row>
@@ -20762,13 +20793,13 @@
         <v>173</v>
       </c>
       <c r="B170" s="2" t="s">
-        <v>1308</v>
+        <v>1310</v>
       </c>
       <c r="C170" s="29" t="s">
-        <v>1309</v>
+        <v>1311</v>
       </c>
       <c r="D170" s="2" t="s">
-        <v>1310</v>
+        <v>1312</v>
       </c>
       <c r="E170" s="30"/>
     </row>
@@ -20777,13 +20808,13 @@
         <v>173</v>
       </c>
       <c r="B171" s="2" t="s">
-        <v>1311</v>
+        <v>1313</v>
       </c>
       <c r="C171" s="31" t="s">
-        <v>1289</v>
+        <v>1291</v>
       </c>
       <c r="D171" s="2" t="s">
-        <v>1265</v>
+        <v>1267</v>
       </c>
       <c r="E171" s="30"/>
     </row>
@@ -20792,13 +20823,13 @@
         <v>804</v>
       </c>
       <c r="B172" s="2" t="s">
-        <v>1312</v>
+        <v>1314</v>
       </c>
       <c r="C172" s="33" t="s">
-        <v>1313</v>
+        <v>1315</v>
       </c>
       <c r="D172" s="2" t="s">
-        <v>1314</v>
+        <v>1316</v>
       </c>
     </row>
     <row r="173" customFormat="false" ht="13" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20806,13 +20837,13 @@
         <v>804</v>
       </c>
       <c r="B173" s="2" t="s">
-        <v>1022</v>
+        <v>1024</v>
       </c>
       <c r="C173" s="33" t="s">
-        <v>1315</v>
+        <v>1317</v>
       </c>
       <c r="D173" s="2" t="s">
-        <v>1024</v>
+        <v>1026</v>
       </c>
     </row>
     <row r="174" customFormat="false" ht="13" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20820,13 +20851,13 @@
         <v>804</v>
       </c>
       <c r="B174" s="2" t="s">
-        <v>1316</v>
+        <v>1318</v>
       </c>
       <c r="C174" s="33" t="s">
-        <v>1317</v>
+        <v>1319</v>
       </c>
       <c r="D174" s="2" t="s">
-        <v>1318</v>
+        <v>1320</v>
       </c>
     </row>
     <row r="175" customFormat="false" ht="13" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20834,13 +20865,13 @@
         <v>804</v>
       </c>
       <c r="B175" s="2" t="s">
-        <v>1080</v>
+        <v>1082</v>
       </c>
       <c r="C175" s="2" t="s">
-        <v>1319</v>
+        <v>1321</v>
       </c>
       <c r="D175" s="2" t="s">
-        <v>1320</v>
+        <v>1322</v>
       </c>
     </row>
     <row r="176" customFormat="false" ht="13" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20848,13 +20879,13 @@
         <v>804</v>
       </c>
       <c r="B176" s="2" t="s">
-        <v>1321</v>
+        <v>1323</v>
       </c>
       <c r="C176" s="31" t="s">
-        <v>1322</v>
+        <v>1324</v>
       </c>
       <c r="D176" s="2" t="s">
-        <v>1265</v>
+        <v>1267</v>
       </c>
     </row>
     <row r="177" customFormat="false" ht="13" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20862,13 +20893,13 @@
         <v>811</v>
       </c>
       <c r="B177" s="2" t="s">
-        <v>1323</v>
+        <v>1325</v>
       </c>
       <c r="C177" s="34" t="s">
-        <v>1324</v>
+        <v>1326</v>
       </c>
       <c r="D177" s="2" t="s">
-        <v>1325</v>
+        <v>1327</v>
       </c>
     </row>
     <row r="178" customFormat="false" ht="13" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20876,13 +20907,13 @@
         <v>811</v>
       </c>
       <c r="B178" s="2" t="s">
-        <v>1326</v>
+        <v>1328</v>
       </c>
       <c r="C178" s="33" t="s">
-        <v>1327</v>
+        <v>1329</v>
       </c>
       <c r="D178" s="2" t="s">
-        <v>1328</v>
+        <v>1330</v>
       </c>
     </row>
     <row r="179" customFormat="false" ht="13" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20890,13 +20921,13 @@
         <v>811</v>
       </c>
       <c r="B179" s="2" t="s">
-        <v>1329</v>
+        <v>1331</v>
       </c>
       <c r="C179" s="33" t="s">
-        <v>1330</v>
+        <v>1332</v>
       </c>
       <c r="D179" s="2" t="s">
-        <v>1331</v>
+        <v>1333</v>
       </c>
     </row>
     <row r="180" customFormat="false" ht="13" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20904,13 +20935,13 @@
         <v>811</v>
       </c>
       <c r="B180" s="2" t="s">
-        <v>1332</v>
+        <v>1334</v>
       </c>
       <c r="C180" s="33" t="s">
-        <v>1333</v>
+        <v>1335</v>
       </c>
       <c r="D180" s="2" t="s">
-        <v>1334</v>
+        <v>1336</v>
       </c>
     </row>
     <row r="181" customFormat="false" ht="13" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20918,13 +20949,13 @@
         <v>811</v>
       </c>
       <c r="B181" s="2" t="s">
-        <v>1335</v>
+        <v>1337</v>
       </c>
       <c r="C181" s="31" t="s">
-        <v>1289</v>
+        <v>1291</v>
       </c>
       <c r="D181" s="2" t="s">
-        <v>1265</v>
+        <v>1267</v>
       </c>
     </row>
     <row r="182" customFormat="false" ht="13" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20932,13 +20963,13 @@
         <v>826</v>
       </c>
       <c r="B182" s="2" t="s">
-        <v>1336</v>
+        <v>1338</v>
       </c>
       <c r="C182" s="29" t="s">
-        <v>1291</v>
+        <v>1293</v>
       </c>
       <c r="D182" s="2" t="s">
-        <v>1337</v>
+        <v>1339</v>
       </c>
     </row>
     <row r="183" customFormat="false" ht="13" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20946,13 +20977,13 @@
         <v>826</v>
       </c>
       <c r="B183" s="2" t="s">
-        <v>1338</v>
+        <v>1340</v>
       </c>
       <c r="C183" s="29" t="s">
-        <v>1294</v>
+        <v>1296</v>
       </c>
       <c r="D183" s="2" t="s">
-        <v>1339</v>
+        <v>1341</v>
       </c>
     </row>
     <row r="184" customFormat="false" ht="13" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20960,13 +20991,13 @@
         <v>826</v>
       </c>
       <c r="B184" s="2" t="s">
-        <v>1340</v>
+        <v>1342</v>
       </c>
       <c r="C184" s="29" t="s">
-        <v>1297</v>
+        <v>1299</v>
       </c>
       <c r="D184" s="2" t="s">
-        <v>1298</v>
+        <v>1300</v>
       </c>
     </row>
     <row r="185" customFormat="false" ht="13" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20974,13 +21005,13 @@
         <v>826</v>
       </c>
       <c r="B185" s="2" t="s">
-        <v>1341</v>
+        <v>1343</v>
       </c>
       <c r="C185" s="29" t="s">
-        <v>1300</v>
+        <v>1302</v>
       </c>
       <c r="D185" s="2" t="s">
-        <v>1301</v>
+        <v>1303</v>
       </c>
     </row>
     <row r="186" customFormat="false" ht="13" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20988,13 +21019,13 @@
         <v>826</v>
       </c>
       <c r="B186" s="2" t="s">
-        <v>1342</v>
+        <v>1344</v>
       </c>
       <c r="C186" s="29" t="s">
-        <v>1303</v>
+        <v>1305</v>
       </c>
       <c r="D186" s="2" t="s">
-        <v>1304</v>
+        <v>1306</v>
       </c>
     </row>
     <row r="187" customFormat="false" ht="13" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21002,13 +21033,13 @@
         <v>826</v>
       </c>
       <c r="B187" s="2" t="s">
-        <v>1343</v>
+        <v>1345</v>
       </c>
       <c r="C187" s="29" t="s">
-        <v>1306</v>
+        <v>1308</v>
       </c>
       <c r="D187" s="2" t="s">
-        <v>1307</v>
+        <v>1309</v>
       </c>
     </row>
     <row r="188" customFormat="false" ht="13" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21016,13 +21047,13 @@
         <v>826</v>
       </c>
       <c r="B188" s="2" t="s">
-        <v>1344</v>
+        <v>1346</v>
       </c>
       <c r="C188" s="29" t="s">
-        <v>1309</v>
+        <v>1311</v>
       </c>
       <c r="D188" s="2" t="s">
-        <v>1310</v>
+        <v>1312</v>
       </c>
     </row>
     <row r="189" customFormat="false" ht="13" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21030,55 +21061,55 @@
         <v>826</v>
       </c>
       <c r="B189" s="2" t="s">
-        <v>1345</v>
+        <v>1347</v>
       </c>
       <c r="C189" s="31" t="s">
-        <v>1322</v>
+        <v>1324</v>
       </c>
       <c r="D189" s="2" t="s">
-        <v>1265</v>
+        <v>1267</v>
       </c>
     </row>
     <row r="190" customFormat="false" ht="13" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A190" s="2" t="s">
-        <v>1346</v>
+        <v>1348</v>
       </c>
       <c r="B190" s="2" t="s">
         <v>139</v>
       </c>
       <c r="C190" s="2" t="s">
-        <v>969</v>
+        <v>971</v>
       </c>
       <c r="D190" s="2" t="s">
-        <v>1347</v>
+        <v>1349</v>
       </c>
     </row>
     <row r="191" customFormat="false" ht="13" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A191" s="2" t="s">
-        <v>1346</v>
+        <v>1348</v>
       </c>
       <c r="B191" s="2" t="s">
-        <v>971</v>
+        <v>973</v>
       </c>
       <c r="C191" s="2" t="s">
-        <v>972</v>
+        <v>974</v>
       </c>
       <c r="D191" s="2" t="s">
-        <v>973</v>
+        <v>975</v>
       </c>
     </row>
     <row r="192" customFormat="false" ht="13" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A192" s="2" t="s">
-        <v>1346</v>
+        <v>1348</v>
       </c>
       <c r="B192" s="2" t="s">
-        <v>1348</v>
+        <v>1350</v>
       </c>
       <c r="C192" s="6" t="s">
-        <v>1322</v>
+        <v>1324</v>
       </c>
       <c r="D192" s="2" t="s">
-        <v>1265</v>
+        <v>1267</v>
       </c>
     </row>
     <row r="193" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21086,13 +21117,13 @@
         <v>184</v>
       </c>
       <c r="B193" s="2" t="s">
-        <v>1349</v>
+        <v>1351</v>
       </c>
       <c r="C193" s="2" t="s">
-        <v>1350</v>
+        <v>1352</v>
       </c>
       <c r="D193" s="44" t="s">
-        <v>1351</v>
+        <v>1353</v>
       </c>
     </row>
     <row r="194" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21100,13 +21131,13 @@
         <v>184</v>
       </c>
       <c r="B194" s="2" t="s">
-        <v>1352</v>
+        <v>1354</v>
       </c>
       <c r="C194" s="2" t="s">
-        <v>1353</v>
+        <v>1355</v>
       </c>
       <c r="D194" s="44" t="s">
-        <v>1354</v>
+        <v>1356</v>
       </c>
     </row>
     <row r="195" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21114,13 +21145,13 @@
         <v>184</v>
       </c>
       <c r="B195" s="2" t="s">
-        <v>1355</v>
+        <v>1357</v>
       </c>
       <c r="C195" s="2" t="s">
-        <v>1356</v>
+        <v>1358</v>
       </c>
       <c r="D195" s="44" t="s">
-        <v>1357</v>
+        <v>1359</v>
       </c>
     </row>
     <row r="196" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21128,13 +21159,13 @@
         <v>184</v>
       </c>
       <c r="B196" s="2" t="s">
-        <v>1358</v>
+        <v>1360</v>
       </c>
       <c r="C196" s="2" t="s">
-        <v>1359</v>
+        <v>1361</v>
       </c>
       <c r="D196" s="44" t="s">
-        <v>1360</v>
+        <v>1362</v>
       </c>
     </row>
     <row r="197" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21142,13 +21173,13 @@
         <v>184</v>
       </c>
       <c r="B197" s="2" t="s">
-        <v>1361</v>
+        <v>1363</v>
       </c>
       <c r="C197" s="2" t="s">
-        <v>1362</v>
+        <v>1364</v>
       </c>
       <c r="D197" s="44" t="s">
-        <v>1363</v>
+        <v>1365</v>
       </c>
     </row>
     <row r="198" customFormat="false" ht="13" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21156,13 +21187,13 @@
         <v>184</v>
       </c>
       <c r="B198" s="2" t="s">
-        <v>1080</v>
+        <v>1082</v>
       </c>
       <c r="C198" s="2" t="s">
-        <v>1081</v>
+        <v>1083</v>
       </c>
       <c r="D198" s="2" t="s">
-        <v>1165</v>
+        <v>1167</v>
       </c>
     </row>
     <row r="199" customFormat="false" ht="13" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21170,181 +21201,181 @@
         <v>184</v>
       </c>
       <c r="B199" s="2" t="s">
-        <v>1348</v>
+        <v>1350</v>
       </c>
       <c r="C199" s="6" t="s">
-        <v>1322</v>
+        <v>1324</v>
       </c>
       <c r="D199" s="2" t="s">
-        <v>1265</v>
+        <v>1267</v>
       </c>
     </row>
     <row r="200" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A200" s="2" t="s">
-        <v>1364</v>
+        <v>1366</v>
       </c>
       <c r="B200" s="2" t="s">
-        <v>1365</v>
+        <v>1367</v>
       </c>
       <c r="C200" s="2" t="s">
-        <v>1366</v>
+        <v>1368</v>
       </c>
       <c r="D200" s="44" t="s">
-        <v>1367</v>
+        <v>1369</v>
       </c>
     </row>
     <row r="201" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A201" s="2" t="s">
-        <v>1364</v>
+        <v>1366</v>
       </c>
       <c r="B201" s="2" t="s">
-        <v>1368</v>
+        <v>1370</v>
       </c>
       <c r="C201" s="2" t="s">
-        <v>1369</v>
+        <v>1371</v>
       </c>
       <c r="D201" s="44" t="s">
-        <v>1370</v>
+        <v>1372</v>
       </c>
     </row>
     <row r="202" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A202" s="2" t="s">
-        <v>1364</v>
+        <v>1366</v>
       </c>
       <c r="B202" s="2" t="s">
-        <v>1371</v>
+        <v>1373</v>
       </c>
       <c r="C202" s="2" t="s">
-        <v>1372</v>
+        <v>1374</v>
       </c>
       <c r="D202" s="44" t="s">
-        <v>1373</v>
+        <v>1375</v>
       </c>
     </row>
     <row r="203" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A203" s="2" t="s">
-        <v>1364</v>
+        <v>1366</v>
       </c>
       <c r="B203" s="2" t="s">
-        <v>1374</v>
+        <v>1376</v>
       </c>
       <c r="C203" s="2" t="s">
-        <v>1375</v>
+        <v>1377</v>
       </c>
       <c r="D203" s="44" t="s">
-        <v>1376</v>
+        <v>1378</v>
       </c>
     </row>
     <row r="204" customFormat="false" ht="13" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A204" s="2" t="s">
-        <v>1364</v>
+        <v>1366</v>
       </c>
       <c r="B204" s="2" t="s">
-        <v>1080</v>
+        <v>1082</v>
       </c>
       <c r="C204" s="2" t="s">
-        <v>1081</v>
+        <v>1083</v>
       </c>
       <c r="D204" s="2" t="s">
-        <v>1165</v>
+        <v>1167</v>
       </c>
     </row>
     <row r="205" customFormat="false" ht="13" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A205" s="2" t="s">
-        <v>1364</v>
+        <v>1366</v>
       </c>
       <c r="B205" s="2" t="s">
-        <v>1348</v>
+        <v>1350</v>
       </c>
       <c r="C205" s="6" t="s">
-        <v>1322</v>
+        <v>1324</v>
       </c>
       <c r="D205" s="2" t="s">
-        <v>1265</v>
+        <v>1267</v>
       </c>
     </row>
     <row r="206" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A206" s="2" t="s">
-        <v>1377</v>
+        <v>1379</v>
       </c>
       <c r="B206" s="2" t="s">
-        <v>1378</v>
+        <v>1380</v>
       </c>
       <c r="C206" s="2" t="s">
-        <v>1379</v>
+        <v>1381</v>
       </c>
       <c r="D206" s="44" t="s">
-        <v>1379</v>
+        <v>1381</v>
       </c>
     </row>
     <row r="207" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A207" s="2" t="s">
-        <v>1377</v>
+        <v>1379</v>
       </c>
       <c r="B207" s="2" t="s">
-        <v>1380</v>
+        <v>1382</v>
       </c>
       <c r="C207" s="2" t="s">
-        <v>1381</v>
+        <v>1383</v>
       </c>
       <c r="D207" s="44" t="s">
-        <v>1382</v>
+        <v>1384</v>
       </c>
     </row>
     <row r="208" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A208" s="2" t="s">
-        <v>1377</v>
+        <v>1379</v>
       </c>
       <c r="B208" s="2" t="s">
-        <v>1383</v>
+        <v>1385</v>
       </c>
       <c r="C208" s="2" t="s">
-        <v>1384</v>
+        <v>1386</v>
       </c>
       <c r="D208" s="44" t="s">
-        <v>1385</v>
+        <v>1387</v>
       </c>
     </row>
     <row r="209" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A209" s="2" t="s">
-        <v>1377</v>
+        <v>1379</v>
       </c>
       <c r="B209" s="2" t="s">
-        <v>1386</v>
+        <v>1388</v>
       </c>
       <c r="C209" s="2" t="s">
-        <v>1387</v>
+        <v>1389</v>
       </c>
       <c r="D209" s="44" t="s">
-        <v>1376</v>
+        <v>1378</v>
       </c>
     </row>
     <row r="210" customFormat="false" ht="13" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A210" s="2" t="s">
-        <v>1377</v>
+        <v>1379</v>
       </c>
       <c r="B210" s="2" t="s">
-        <v>1080</v>
+        <v>1082</v>
       </c>
       <c r="C210" s="2" t="s">
-        <v>1081</v>
+        <v>1083</v>
       </c>
       <c r="D210" s="2" t="s">
-        <v>1165</v>
+        <v>1167</v>
       </c>
     </row>
     <row r="211" customFormat="false" ht="13" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A211" s="2" t="s">
-        <v>1377</v>
+        <v>1379</v>
       </c>
       <c r="B211" s="2" t="s">
-        <v>1348</v>
+        <v>1350</v>
       </c>
       <c r="C211" s="6" t="s">
-        <v>1322</v>
+        <v>1324</v>
       </c>
       <c r="D211" s="2" t="s">
-        <v>1265</v>
+        <v>1267</v>
       </c>
     </row>
     <row r="212" customFormat="false" ht="13" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21352,13 +21383,13 @@
         <v>286</v>
       </c>
       <c r="B212" s="2" t="s">
-        <v>1388</v>
+        <v>1390</v>
       </c>
       <c r="C212" s="2" t="s">
-        <v>859</v>
+        <v>860</v>
       </c>
       <c r="D212" s="2" t="s">
-        <v>1389</v>
+        <v>1391</v>
       </c>
     </row>
     <row r="213" customFormat="false" ht="13" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21366,13 +21397,13 @@
         <v>286</v>
       </c>
       <c r="B213" s="2" t="s">
-        <v>1390</v>
+        <v>1392</v>
       </c>
       <c r="C213" s="12" t="s">
-        <v>863</v>
+        <v>864</v>
       </c>
       <c r="D213" s="2" t="s">
-        <v>864</v>
+        <v>865</v>
       </c>
     </row>
     <row r="214" customFormat="false" ht="13" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21380,13 +21411,13 @@
         <v>286</v>
       </c>
       <c r="B214" s="2" t="s">
-        <v>1391</v>
+        <v>1393</v>
       </c>
       <c r="C214" s="12" t="s">
-        <v>867</v>
+        <v>868</v>
       </c>
       <c r="D214" s="2" t="s">
-        <v>868</v>
+        <v>869</v>
       </c>
     </row>
     <row r="215" customFormat="false" ht="13" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21394,13 +21425,13 @@
         <v>286</v>
       </c>
       <c r="B215" s="2" t="s">
-        <v>1392</v>
+        <v>1394</v>
       </c>
       <c r="C215" s="12" t="s">
-        <v>871</v>
+        <v>872</v>
       </c>
       <c r="D215" s="2" t="s">
-        <v>872</v>
+        <v>873</v>
       </c>
     </row>
     <row r="216" customFormat="false" ht="13" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21408,13 +21439,13 @@
         <v>286</v>
       </c>
       <c r="B216" s="2" t="s">
-        <v>1393</v>
+        <v>1395</v>
       </c>
       <c r="C216" s="12" t="s">
-        <v>875</v>
+        <v>876</v>
       </c>
       <c r="D216" s="2" t="s">
-        <v>876</v>
+        <v>877</v>
       </c>
     </row>
     <row r="217" customFormat="false" ht="13" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21422,10 +21453,10 @@
         <v>286</v>
       </c>
       <c r="B217" s="2" t="s">
-        <v>1394</v>
+        <v>1396</v>
       </c>
       <c r="C217" s="2" t="s">
-        <v>879</v>
+        <v>880</v>
       </c>
       <c r="D217" s="2" t="s">
         <v>457</v>
@@ -21439,10 +21470,10 @@
         <v>391</v>
       </c>
       <c r="C218" s="12" t="s">
-        <v>882</v>
+        <v>883</v>
       </c>
       <c r="D218" s="2" t="s">
-        <v>883</v>
+        <v>884</v>
       </c>
     </row>
     <row r="219" customFormat="false" ht="13" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21450,83 +21481,83 @@
         <v>286</v>
       </c>
       <c r="B219" s="2" t="s">
-        <v>1013</v>
+        <v>1015</v>
       </c>
       <c r="C219" s="2" t="s">
-        <v>1014</v>
+        <v>1016</v>
       </c>
       <c r="D219" s="2" t="s">
-        <v>1015</v>
+        <v>1017</v>
       </c>
     </row>
     <row r="220" customFormat="false" ht="13" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A220" s="45" t="s">
-        <v>1395</v>
+        <v>1397</v>
       </c>
       <c r="B220" s="2" t="s">
-        <v>900</v>
+        <v>902</v>
       </c>
       <c r="C220" s="2" t="s">
-        <v>901</v>
+        <v>903</v>
       </c>
       <c r="D220" s="2" t="s">
-        <v>902</v>
+        <v>904</v>
       </c>
     </row>
     <row r="221" customFormat="false" ht="13" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A221" s="45" t="s">
-        <v>1395</v>
+        <v>1397</v>
       </c>
       <c r="B221" s="2" t="s">
-        <v>904</v>
+        <v>906</v>
       </c>
       <c r="C221" s="2" t="s">
-        <v>905</v>
+        <v>907</v>
       </c>
       <c r="D221" s="2" t="s">
-        <v>906</v>
+        <v>908</v>
       </c>
     </row>
     <row r="222" customFormat="false" ht="13" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A222" s="45" t="s">
-        <v>1395</v>
+        <v>1397</v>
       </c>
       <c r="B222" s="2" t="s">
-        <v>908</v>
+        <v>910</v>
       </c>
       <c r="C222" s="12" t="s">
-        <v>909</v>
+        <v>911</v>
       </c>
       <c r="D222" s="2" t="s">
-        <v>910</v>
+        <v>912</v>
       </c>
     </row>
     <row r="223" customFormat="false" ht="13" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A223" s="45" t="s">
-        <v>1395</v>
+        <v>1397</v>
       </c>
       <c r="B223" s="2" t="s">
-        <v>912</v>
+        <v>914</v>
       </c>
       <c r="C223" s="2" t="s">
-        <v>913</v>
+        <v>915</v>
       </c>
       <c r="D223" s="2" t="s">
-        <v>914</v>
+        <v>916</v>
       </c>
     </row>
     <row r="224" customFormat="false" ht="13" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A224" s="4" t="s">
-        <v>1395</v>
+        <v>1397</v>
       </c>
       <c r="B224" s="2" t="s">
-        <v>1013</v>
+        <v>1015</v>
       </c>
       <c r="C224" s="2" t="s">
-        <v>1014</v>
+        <v>1016</v>
       </c>
       <c r="D224" s="2" t="s">
-        <v>1015</v>
+        <v>1017</v>
       </c>
     </row>
     <row r="225" customFormat="false" ht="13" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21534,13 +21565,13 @@
         <v>679</v>
       </c>
       <c r="B225" s="2" t="s">
-        <v>1396</v>
+        <v>1398</v>
       </c>
       <c r="C225" s="2" t="s">
-        <v>1397</v>
+        <v>1399</v>
       </c>
       <c r="D225" s="2" t="s">
-        <v>1398</v>
+        <v>1400</v>
       </c>
     </row>
     <row r="226" customFormat="false" ht="13" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21548,13 +21579,13 @@
         <v>679</v>
       </c>
       <c r="B226" s="2" t="s">
-        <v>1399</v>
+        <v>1401</v>
       </c>
       <c r="C226" s="2" t="s">
-        <v>1400</v>
+        <v>1402</v>
       </c>
       <c r="D226" s="2" t="s">
-        <v>1401</v>
+        <v>1403</v>
       </c>
     </row>
     <row r="227" customFormat="false" ht="13" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21562,13 +21593,13 @@
         <v>679</v>
       </c>
       <c r="B227" s="2" t="s">
-        <v>1402</v>
+        <v>1404</v>
       </c>
       <c r="C227" s="2" t="s">
-        <v>1403</v>
+        <v>1405</v>
       </c>
       <c r="D227" s="2" t="s">
-        <v>1404</v>
+        <v>1406</v>
       </c>
     </row>
     <row r="228" customFormat="false" ht="13" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21576,13 +21607,13 @@
         <v>679</v>
       </c>
       <c r="B228" s="2" t="s">
-        <v>1405</v>
+        <v>1407</v>
       </c>
       <c r="C228" s="2" t="s">
-        <v>1406</v>
+        <v>1408</v>
       </c>
       <c r="D228" s="2" t="s">
-        <v>1407</v>
+        <v>1409</v>
       </c>
     </row>
     <row r="229" customFormat="false" ht="13" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21590,13 +21621,13 @@
         <v>415</v>
       </c>
       <c r="B229" s="2" t="s">
-        <v>1408</v>
+        <v>1410</v>
       </c>
       <c r="C229" s="2" t="s">
-        <v>1409</v>
+        <v>1411</v>
       </c>
       <c r="D229" s="2" t="s">
-        <v>1410</v>
+        <v>1412</v>
       </c>
     </row>
     <row r="230" customFormat="false" ht="13" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21604,13 +21635,13 @@
         <v>415</v>
       </c>
       <c r="B230" s="2" t="s">
-        <v>1411</v>
+        <v>1413</v>
       </c>
       <c r="C230" s="2" t="s">
-        <v>1412</v>
+        <v>1414</v>
       </c>
       <c r="D230" s="2" t="s">
-        <v>1413</v>
+        <v>1415</v>
       </c>
     </row>
     <row r="231" customFormat="false" ht="13" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21621,10 +21652,10 @@
         <v>139</v>
       </c>
       <c r="C231" s="2" t="s">
-        <v>969</v>
+        <v>971</v>
       </c>
       <c r="D231" s="2" t="s">
-        <v>1414</v>
+        <v>1416</v>
       </c>
     </row>
     <row r="232" customFormat="false" ht="13" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21632,13 +21663,13 @@
         <v>332</v>
       </c>
       <c r="B232" s="2" t="s">
-        <v>1415</v>
+        <v>1417</v>
       </c>
       <c r="C232" s="2" t="s">
-        <v>1416</v>
+        <v>1418</v>
       </c>
       <c r="D232" s="2" t="s">
-        <v>1417</v>
+        <v>1419</v>
       </c>
     </row>
     <row r="233" customFormat="false" ht="13" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21646,13 +21677,13 @@
         <v>332</v>
       </c>
       <c r="B233" s="2" t="s">
-        <v>1418</v>
+        <v>1420</v>
       </c>
       <c r="C233" s="2" t="s">
-        <v>1419</v>
+        <v>1421</v>
       </c>
       <c r="D233" s="2" t="s">
-        <v>1420</v>
+        <v>1422</v>
       </c>
     </row>
     <row r="234" customFormat="false" ht="13" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21660,13 +21691,13 @@
         <v>332</v>
       </c>
       <c r="B234" s="2" t="s">
-        <v>1421</v>
+        <v>1423</v>
       </c>
       <c r="C234" s="2" t="s">
-        <v>1422</v>
+        <v>1424</v>
       </c>
       <c r="D234" s="2" t="s">
-        <v>1423</v>
+        <v>1425</v>
       </c>
     </row>
   </sheetData>
@@ -21694,39 +21725,39 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="42" t="s">
-        <v>1424</v>
+        <v>1426</v>
       </c>
       <c r="B1" s="42" t="s">
-        <v>1425</v>
+        <v>1427</v>
       </c>
       <c r="C1" s="42" t="s">
-        <v>1426</v>
+        <v>1428</v>
       </c>
       <c r="D1" s="42" t="s">
-        <v>1427</v>
+        <v>1429</v>
       </c>
       <c r="E1" s="42" t="s">
-        <v>1428</v>
+        <v>1430</v>
       </c>
       <c r="F1" s="42" t="s">
-        <v>1429</v>
+        <v>1431</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="14.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="43" t="s">
-        <v>1430</v>
+        <v>1432</v>
       </c>
       <c r="B2" s="43" t="s">
-        <v>1431</v>
+        <v>1433</v>
       </c>
       <c r="C2" s="46" t="s">
-        <v>1432</v>
+        <v>1434</v>
       </c>
       <c r="D2" s="43" t="s">
-        <v>1433</v>
+        <v>1435</v>
       </c>
       <c r="E2" s="43" t="s">
-        <v>1434</v>
+        <v>1436</v>
       </c>
       <c r="F2" s="43"/>
     </row>

</xml_diff>